<commit_message>
Add Record Splits to the members-only /bets board.
sj bets now reads the Record Splits sheet by header names (Bettor, Source
tab, Class, Sport) instead of fixed ranges, writes record_splits.json, and
tolerates the new Bets Pick Class column. Lockedin_Sportz (Z-) is mapped
like LC; any P/L for him is labeled hypothetical 1u because he posts no
stake or units. The portal adds a Record splits tab with fade highlighting.

Co-authored-by: Austin Wiley <thejayer@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/bets/tracker_tabs.xlsx
+++ b/tests/fixtures/bets/tracker_tabs.xlsx
@@ -6,12 +6,13 @@
     <sheet name="Parlay Legs" sheetId="2" r:id="rId2"/>
     <sheet name="BetMGM Public Warnings" sheetId="3" r:id="rId3"/>
     <sheet name="Summary" sheetId="4" r:id="rId4"/>
+    <sheet name="Record Splits" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="848">
   <si>
     <t>Bet ID</t>
   </si>
@@ -103,6 +104,9 @@
     <t>Settled units (helper)</t>
   </si>
   <si>
+    <t>Pick Class</t>
+  </si>
+  <si>
     <t>Extra unused</t>
   </si>
   <si>
@@ -166,6 +170,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -226,6 +233,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -286,6 +296,9 @@
     <t>Parlay/multi-leg</t>
   </si>
   <si>
+    <t>Parlay</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -349,6 +362,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -409,6 +425,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -469,6 +488,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -529,6 +551,9 @@
     <t>Parlay/multi-leg</t>
   </si>
   <si>
+    <t>Parlay</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -592,6 +617,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Prop</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -652,6 +680,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -715,9 +746,132 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
+    <t>Z-1</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>2026-09-18 12:00:00</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>8:20 PM</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>player prop</t>
+  </si>
+  <si>
+    <t>Mahomes over 249.5 pass yds</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>graded</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>https://x.com/Lockedin_Sportz/status/1</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>ignore-me</t>
+  </si>
+  <si>
+    <t>Z-2</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>2026-09-18 12:00:00</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>8:20 PM</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>player prop</t>
+  </si>
+  <si>
+    <t>Kelce over 59.5 rec yds</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>graded</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>https://x.com/Lockedin_Sportz/status/1</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>ignore-me</t>
+  </si>
+  <si>
     <t>Leg ID</t>
   </si>
   <si>
@@ -1955,6 +2109,453 @@
   </si>
   <si>
     <t>do not read</t>
+  </si>
+  <si>
+    <t>Record Splits</t>
+  </si>
+  <si>
+    <t>Synthetic fixture — not live data</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Win %</t>
+  </si>
+  <si>
+    <t>Bettor</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Source tab</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Posted units P&amp;L</t>
+  </si>
+  <si>
+    <t>$ P&amp;L</t>
+  </si>
+  <si>
+    <t>$ staked</t>
+  </si>
+  <si>
+    <t>Flat 1u</t>
+  </si>
+  <si>
+    <t>1u fade at -110</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>chellgod</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>chellgod</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>chellgod</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>btidy216</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>btidy216</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>btidy216</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>@Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Bets W vs splits</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Parlay legs vs splits</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Sport split</t>
+  </si>
+  <si>
+    <t>Sport</t>
+  </si>
+  <si>
+    <t>Bettor</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Source tab</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Win %</t>
+  </si>
+  <si>
+    <t>1u fade at -110</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>CFB</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>MLB</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>CFB</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
   </si>
 </sst>
 </file>
@@ -2081,55 +2682,58 @@
       <c r="AE1" t="s">
         <v>30</v>
       </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P2" t="n">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="Q2" t="n">
         <v>100</v>
@@ -2139,77 +2743,80 @@
         <v>100</v>
       </c>
       <c r="T2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="U2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="V2"/>
       <c r="W2"/>
       <c r="X2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Y2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Z2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AA2"/>
       <c r="AB2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AC2" t="n">
         <v>100</v>
       </c>
       <c r="AD2"/>
       <c r="AE2" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I3"/>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="P3" t="n">
         <v>1.909</v>
@@ -2224,25 +2831,25 @@
         <v>100</v>
       </c>
       <c r="T3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="U3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="V3"/>
       <c r="W3"/>
       <c r="X3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Y3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Z3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AA3"/>
       <c r="AB3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="AC3" t="n">
         <v>110</v>
@@ -2251,55 +2858,58 @@
         <v>1</v>
       </c>
       <c r="AE3" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I4"/>
       <c r="J4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="L4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="M4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="N4" t="n">
         <v>2</v>
       </c>
       <c r="O4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="P4" t="n">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="Q4" t="n">
         <v>50</v>
@@ -2309,79 +2919,82 @@
         <v>150</v>
       </c>
       <c r="T4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="U4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="V4"/>
       <c r="W4"/>
       <c r="X4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="Y4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="Z4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="AA4"/>
       <c r="AB4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="AC4" t="n">
         <v>50</v>
       </c>
       <c r="AD4"/>
       <c r="AE4" t="s">
-        <v>91</v>
+        <v>94</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="K5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="M5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="P5" t="n">
         <v>2.5</v>
@@ -2394,77 +3007,80 @@
         <v>2500</v>
       </c>
       <c r="T5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="U5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="V5"/>
       <c r="W5"/>
       <c r="X5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="Y5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="Z5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="AA5"/>
       <c r="AB5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="AC5" t="n">
         <v>1000</v>
       </c>
       <c r="AD5"/>
       <c r="AE5" t="s">
-        <v>112</v>
+        <v>116</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E6" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="G6" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I6"/>
       <c r="J6" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="K6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="L6" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="M6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="P6" t="n">
         <v>1.909</v>
@@ -2477,77 +3093,80 @@
         <v>1818</v>
       </c>
       <c r="T6" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="U6" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="V6"/>
       <c r="W6"/>
       <c r="X6" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="Y6" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="Z6" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="AA6"/>
       <c r="AB6" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="AC6" t="n">
         <v>2000</v>
       </c>
       <c r="AD6"/>
       <c r="AE6" t="s">
-        <v>132</v>
+        <v>137</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E7" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G7" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="H7" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="I7"/>
       <c r="J7" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="K7" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="L7" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="M7" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="P7" t="n">
         <v>1.5</v>
@@ -2560,77 +3179,80 @@
         <v>200</v>
       </c>
       <c r="T7" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="U7" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="V7"/>
       <c r="W7"/>
       <c r="X7" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="Y7" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="Z7" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="AA7"/>
       <c r="AB7" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="AC7" t="n">
         <v>400</v>
       </c>
       <c r="AD7"/>
       <c r="AE7" t="s">
-        <v>152</v>
+        <v>158</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B8" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C8" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D8" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E8" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="F8" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="G8" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="H8" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="I8"/>
       <c r="J8" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="K8" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="L8" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="M8" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="N8" t="n">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="P8" t="n">
         <v>3.5</v>
@@ -2643,79 +3265,82 @@
         <v>100</v>
       </c>
       <c r="T8" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="U8" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="V8"/>
       <c r="W8"/>
       <c r="X8" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="Y8" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="Z8" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="AA8"/>
       <c r="AB8" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="AC8" t="n">
         <v>40</v>
       </c>
       <c r="AD8"/>
       <c r="AE8" t="s">
-        <v>172</v>
+        <v>179</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="E9" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="F9" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="G9" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="H9" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="I9" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="J9" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="K9" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="L9" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="M9" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="N9" t="n">
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="P9" t="n">
         <v>1.833</v>
@@ -2728,77 +3353,80 @@
         <v>50</v>
       </c>
       <c r="T9" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="U9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="V9"/>
       <c r="W9"/>
       <c r="X9" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="Y9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="Z9" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="AA9"/>
       <c r="AB9" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="AC9" t="n">
         <v>60</v>
       </c>
       <c r="AD9"/>
       <c r="AE9" t="s">
-        <v>193</v>
+        <v>201</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B10" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="C10" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="D10" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="E10" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="F10" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="G10" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="H10" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="I10"/>
       <c r="J10" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="K10" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="L10" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="M10" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="N10" t="n">
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="P10" t="n">
         <v>1.667</v>
@@ -2811,79 +3439,82 @@
         <v>20</v>
       </c>
       <c r="T10" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="U10" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="V10"/>
       <c r="W10"/>
       <c r="X10" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="Y10" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="Z10" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="AA10"/>
       <c r="AB10" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="AC10" t="n">
         <v>30</v>
       </c>
       <c r="AD10"/>
       <c r="AE10" t="s">
-        <v>213</v>
+        <v>222</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B11" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="C11" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="D11" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="E11" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="F11" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="G11" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="H11" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="I11" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="J11" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="K11" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="L11" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="M11" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="N11" t="n">
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="P11" t="n">
         <v>1.909</v>
@@ -2896,32 +3527,187 @@
         <v>18.18</v>
       </c>
       <c r="T11" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="U11" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="V11"/>
       <c r="W11"/>
       <c r="X11" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="Y11" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="Z11" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="AA11"/>
       <c r="AB11" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="AC11" t="n">
         <v>20</v>
       </c>
       <c r="AD11"/>
       <c r="AE11" t="s">
-        <v>234</v>
+        <v>244</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D12" t="s">
+        <v>249</v>
+      </c>
+      <c r="E12" t="s">
+        <v>250</v>
+      </c>
+      <c r="F12" t="s">
+        <v>251</v>
+      </c>
+      <c r="G12" t="s">
+        <v>252</v>
+      </c>
+      <c r="H12" t="s">
+        <v>253</v>
+      </c>
+      <c r="I12"/>
+      <c r="J12" t="s">
+        <v>254</v>
+      </c>
+      <c r="K12" t="s">
+        <v>255</v>
+      </c>
+      <c r="L12" t="s">
+        <v>256</v>
+      </c>
+      <c r="M12" t="s">
+        <v>257</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12" t="s">
+        <v>258</v>
+      </c>
+      <c r="U12" t="s">
+        <v>259</v>
+      </c>
+      <c r="V12"/>
+      <c r="W12"/>
+      <c r="X12" t="s">
+        <v>260</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>261</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>262</v>
+      </c>
+      <c r="AA12"/>
+      <c r="AB12" t="s">
+        <v>263</v>
+      </c>
+      <c r="AC12"/>
+      <c r="AD12"/>
+      <c r="AE12" t="s">
+        <v>264</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B13" t="s">
+        <v>267</v>
+      </c>
+      <c r="C13" t="s">
+        <v>268</v>
+      </c>
+      <c r="D13" t="s">
+        <v>269</v>
+      </c>
+      <c r="E13" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G13" t="s">
+        <v>272</v>
+      </c>
+      <c r="H13" t="s">
+        <v>273</v>
+      </c>
+      <c r="I13"/>
+      <c r="J13" t="s">
+        <v>274</v>
+      </c>
+      <c r="K13" t="s">
+        <v>275</v>
+      </c>
+      <c r="L13" t="s">
+        <v>276</v>
+      </c>
+      <c r="M13" t="s">
+        <v>277</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13" t="s">
+        <v>278</v>
+      </c>
+      <c r="U13" t="s">
+        <v>279</v>
+      </c>
+      <c r="V13"/>
+      <c r="W13"/>
+      <c r="X13" t="s">
+        <v>280</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>281</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>282</v>
+      </c>
+      <c r="AA13"/>
+      <c r="AB13" t="s">
+        <v>283</v>
+      </c>
+      <c r="AC13"/>
+      <c r="AD13"/>
+      <c r="AE13" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -2933,178 +3719,178 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>235</v>
+        <v>286</v>
       </c>
       <c r="B1" t="s">
-        <v>236</v>
+        <v>287</v>
       </c>
       <c r="C1" t="s">
-        <v>237</v>
+        <v>288</v>
       </c>
       <c r="D1" t="s">
-        <v>238</v>
+        <v>289</v>
       </c>
       <c r="E1" t="s">
-        <v>239</v>
+        <v>290</v>
       </c>
       <c r="F1" t="s">
-        <v>240</v>
+        <v>291</v>
       </c>
       <c r="G1" t="s">
-        <v>241</v>
+        <v>292</v>
       </c>
       <c r="H1" t="s">
-        <v>242</v>
+        <v>293</v>
       </c>
       <c r="I1" t="s">
-        <v>243</v>
+        <v>294</v>
       </c>
       <c r="J1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="K1" t="s">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="L1" t="s">
-        <v>246</v>
+        <v>297</v>
       </c>
       <c r="M1" t="s">
-        <v>247</v>
+        <v>298</v>
       </c>
       <c r="N1" t="s">
-        <v>248</v>
+        <v>299</v>
       </c>
       <c r="O1" t="s">
-        <v>249</v>
+        <v>300</v>
       </c>
       <c r="P1" t="s">
-        <v>250</v>
+        <v>301</v>
       </c>
       <c r="Q1" t="s">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="R1" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="S1" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
       <c r="T1" t="s">
-        <v>254</v>
+        <v>305</v>
       </c>
       <c r="U1" t="s">
-        <v>255</v>
+        <v>306</v>
       </c>
       <c r="V1" t="s">
-        <v>256</v>
+        <v>307</v>
       </c>
       <c r="W1" t="s">
-        <v>257</v>
+        <v>308</v>
       </c>
       <c r="X1" t="s">
-        <v>258</v>
+        <v>309</v>
       </c>
       <c r="Y1" t="s">
-        <v>259</v>
+        <v>310</v>
       </c>
       <c r="Z1" t="s">
-        <v>260</v>
+        <v>311</v>
       </c>
       <c r="AA1" t="s">
-        <v>261</v>
+        <v>312</v>
       </c>
       <c r="AB1" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="AC1" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
       <c r="AD1" t="s">
-        <v>264</v>
+        <v>315</v>
       </c>
       <c r="AE1" t="s">
-        <v>265</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>266</v>
+        <v>317</v>
       </c>
       <c r="B2" t="s">
-        <v>267</v>
+        <v>318</v>
       </c>
       <c r="C2" t="s">
-        <v>268</v>
+        <v>319</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>269</v>
+        <v>320</v>
       </c>
       <c r="F2" t="s">
-        <v>270</v>
+        <v>321</v>
       </c>
       <c r="G2" t="s">
-        <v>271</v>
+        <v>322</v>
       </c>
       <c r="H2" t="s">
-        <v>272</v>
+        <v>323</v>
       </c>
       <c r="I2" t="s">
-        <v>273</v>
+        <v>324</v>
       </c>
       <c r="J2" t="s">
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="K2" t="s">
-        <v>275</v>
+        <v>326</v>
       </c>
       <c r="L2" t="s">
-        <v>276</v>
+        <v>327</v>
       </c>
       <c r="M2" t="s">
-        <v>277</v>
+        <v>328</v>
       </c>
       <c r="N2" t="s">
-        <v>278</v>
+        <v>329</v>
       </c>
       <c r="O2" t="s">
-        <v>279</v>
+        <v>330</v>
       </c>
       <c r="P2" t="s">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="Q2" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="R2"/>
       <c r="S2" t="s">
-        <v>282</v>
+        <v>333</v>
       </c>
       <c r="T2" t="s">
-        <v>283</v>
+        <v>334</v>
       </c>
       <c r="U2" t="s">
-        <v>284</v>
+        <v>335</v>
       </c>
       <c r="V2" t="s">
-        <v>285</v>
+        <v>336</v>
       </c>
       <c r="W2" t="s">
-        <v>286</v>
+        <v>337</v>
       </c>
       <c r="X2" t="s">
-        <v>287</v>
+        <v>338</v>
       </c>
       <c r="Y2" t="s">
-        <v>288</v>
+        <v>339</v>
       </c>
       <c r="Z2" t="s">
-        <v>289</v>
+        <v>340</v>
       </c>
       <c r="AA2" t="s">
-        <v>290</v>
+        <v>341</v>
       </c>
       <c r="AB2" t="n">
         <v>2</v>
@@ -3113,93 +3899,93 @@
         <v>1</v>
       </c>
       <c r="AD2" t="s">
-        <v>291</v>
+        <v>342</v>
       </c>
       <c r="AE2" t="s">
-        <v>292</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>293</v>
+        <v>344</v>
       </c>
       <c r="B3" t="s">
-        <v>294</v>
+        <v>345</v>
       </c>
       <c r="C3" t="s">
-        <v>295</v>
+        <v>346</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>296</v>
+        <v>347</v>
       </c>
       <c r="F3" t="s">
-        <v>297</v>
+        <v>348</v>
       </c>
       <c r="G3" t="s">
-        <v>298</v>
+        <v>349</v>
       </c>
       <c r="H3" t="s">
-        <v>299</v>
+        <v>350</v>
       </c>
       <c r="I3" t="s">
-        <v>300</v>
+        <v>351</v>
       </c>
       <c r="J3" t="s">
-        <v>301</v>
+        <v>352</v>
       </c>
       <c r="K3" t="s">
-        <v>302</v>
+        <v>353</v>
       </c>
       <c r="L3" t="s">
-        <v>303</v>
+        <v>354</v>
       </c>
       <c r="M3" t="s">
-        <v>304</v>
+        <v>355</v>
       </c>
       <c r="N3" t="s">
-        <v>305</v>
+        <v>356</v>
       </c>
       <c r="O3" t="s">
-        <v>306</v>
+        <v>357</v>
       </c>
       <c r="P3" t="s">
-        <v>307</v>
+        <v>358</v>
       </c>
       <c r="Q3" t="s">
-        <v>308</v>
+        <v>359</v>
       </c>
       <c r="R3" t="s">
-        <v>309</v>
+        <v>360</v>
       </c>
       <c r="S3" t="s">
-        <v>310</v>
+        <v>361</v>
       </c>
       <c r="T3" t="s">
-        <v>311</v>
+        <v>362</v>
       </c>
       <c r="U3" t="s">
-        <v>312</v>
+        <v>363</v>
       </c>
       <c r="V3" t="s">
-        <v>313</v>
+        <v>364</v>
       </c>
       <c r="W3" t="s">
-        <v>314</v>
+        <v>365</v>
       </c>
       <c r="X3" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
       <c r="Y3" t="s">
-        <v>316</v>
+        <v>367</v>
       </c>
       <c r="Z3" t="s">
-        <v>317</v>
+        <v>368</v>
       </c>
       <c r="AA3" t="s">
-        <v>318</v>
+        <v>369</v>
       </c>
       <c r="AB3" t="n">
         <v>2</v>
@@ -3208,91 +3994,91 @@
         <v>1</v>
       </c>
       <c r="AD3" t="s">
-        <v>319</v>
+        <v>370</v>
       </c>
       <c r="AE3" t="s">
-        <v>320</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>321</v>
+        <v>372</v>
       </c>
       <c r="B4" t="s">
-        <v>322</v>
+        <v>373</v>
       </c>
       <c r="C4" t="s">
-        <v>323</v>
+        <v>374</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="F4" t="s">
-        <v>325</v>
+        <v>376</v>
       </c>
       <c r="G4" t="s">
-        <v>326</v>
+        <v>377</v>
       </c>
       <c r="H4" t="s">
-        <v>327</v>
+        <v>378</v>
       </c>
       <c r="I4" t="s">
-        <v>328</v>
+        <v>379</v>
       </c>
       <c r="J4" t="s">
-        <v>329</v>
+        <v>380</v>
       </c>
       <c r="K4" t="s">
-        <v>330</v>
+        <v>381</v>
       </c>
       <c r="L4" t="s">
-        <v>331</v>
+        <v>382</v>
       </c>
       <c r="M4" t="s">
-        <v>332</v>
+        <v>383</v>
       </c>
       <c r="N4" t="s">
-        <v>333</v>
+        <v>384</v>
       </c>
       <c r="O4" t="s">
-        <v>334</v>
+        <v>385</v>
       </c>
       <c r="P4" t="s">
-        <v>335</v>
+        <v>386</v>
       </c>
       <c r="Q4" t="s">
-        <v>336</v>
+        <v>387</v>
       </c>
       <c r="R4"/>
       <c r="S4" t="s">
-        <v>337</v>
+        <v>388</v>
       </c>
       <c r="T4" t="s">
-        <v>338</v>
+        <v>389</v>
       </c>
       <c r="U4" t="s">
-        <v>339</v>
+        <v>390</v>
       </c>
       <c r="V4" t="s">
-        <v>340</v>
+        <v>391</v>
       </c>
       <c r="W4" t="s">
-        <v>341</v>
+        <v>392</v>
       </c>
       <c r="X4" t="s">
-        <v>342</v>
+        <v>393</v>
       </c>
       <c r="Y4" t="s">
-        <v>343</v>
+        <v>394</v>
       </c>
       <c r="Z4" t="s">
-        <v>344</v>
+        <v>395</v>
       </c>
       <c r="AA4" t="s">
-        <v>345</v>
+        <v>396</v>
       </c>
       <c r="AB4" t="n">
         <v>2</v>
@@ -3301,91 +4087,91 @@
         <v>1</v>
       </c>
       <c r="AD4" t="s">
-        <v>346</v>
+        <v>397</v>
       </c>
       <c r="AE4" t="s">
-        <v>347</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>348</v>
+        <v>399</v>
       </c>
       <c r="B5" t="s">
-        <v>349</v>
+        <v>400</v>
       </c>
       <c r="C5" t="s">
-        <v>350</v>
+        <v>401</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>351</v>
+        <v>402</v>
       </c>
       <c r="F5" t="s">
-        <v>352</v>
+        <v>403</v>
       </c>
       <c r="G5" t="s">
-        <v>353</v>
+        <v>404</v>
       </c>
       <c r="H5" t="s">
-        <v>354</v>
+        <v>405</v>
       </c>
       <c r="I5" t="s">
-        <v>355</v>
+        <v>406</v>
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>356</v>
+        <v>407</v>
       </c>
       <c r="L5" t="s">
-        <v>357</v>
+        <v>408</v>
       </c>
       <c r="M5" t="s">
-        <v>358</v>
+        <v>409</v>
       </c>
       <c r="N5" t="s">
-        <v>359</v>
+        <v>410</v>
       </c>
       <c r="O5" t="s">
-        <v>360</v>
+        <v>411</v>
       </c>
       <c r="P5" t="s">
-        <v>361</v>
+        <v>412</v>
       </c>
       <c r="Q5" t="s">
-        <v>362</v>
+        <v>413</v>
       </c>
       <c r="R5" t="s">
-        <v>363</v>
+        <v>414</v>
       </c>
       <c r="S5" t="s">
-        <v>364</v>
+        <v>415</v>
       </c>
       <c r="T5" t="s">
-        <v>365</v>
+        <v>416</v>
       </c>
       <c r="U5" t="s">
-        <v>366</v>
+        <v>417</v>
       </c>
       <c r="V5" t="s">
-        <v>367</v>
+        <v>418</v>
       </c>
       <c r="W5" t="s">
-        <v>368</v>
+        <v>419</v>
       </c>
       <c r="X5" t="s">
-        <v>369</v>
+        <v>420</v>
       </c>
       <c r="Y5" t="s">
-        <v>370</v>
+        <v>421</v>
       </c>
       <c r="Z5" t="s">
-        <v>371</v>
+        <v>422</v>
       </c>
       <c r="AA5" t="s">
-        <v>372</v>
+        <v>423</v>
       </c>
       <c r="AB5" t="n">
         <v>2</v>
@@ -3394,93 +4180,93 @@
         <v>1</v>
       </c>
       <c r="AD5" t="s">
-        <v>373</v>
+        <v>424</v>
       </c>
       <c r="AE5" t="s">
-        <v>374</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>375</v>
+        <v>426</v>
       </c>
       <c r="B6" t="s">
-        <v>376</v>
+        <v>427</v>
       </c>
       <c r="C6" t="s">
-        <v>377</v>
+        <v>428</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>378</v>
+        <v>429</v>
       </c>
       <c r="F6" t="s">
-        <v>379</v>
+        <v>430</v>
       </c>
       <c r="G6" t="s">
-        <v>380</v>
+        <v>431</v>
       </c>
       <c r="H6" t="s">
-        <v>381</v>
+        <v>432</v>
       </c>
       <c r="I6" t="s">
-        <v>382</v>
+        <v>433</v>
       </c>
       <c r="J6" t="s">
-        <v>383</v>
+        <v>434</v>
       </c>
       <c r="K6" t="s">
-        <v>384</v>
+        <v>435</v>
       </c>
       <c r="L6" t="s">
-        <v>385</v>
+        <v>436</v>
       </c>
       <c r="M6" t="s">
-        <v>386</v>
+        <v>437</v>
       </c>
       <c r="N6" t="s">
-        <v>387</v>
+        <v>438</v>
       </c>
       <c r="O6" t="s">
-        <v>388</v>
+        <v>439</v>
       </c>
       <c r="P6" t="s">
-        <v>389</v>
+        <v>440</v>
       </c>
       <c r="Q6" t="s">
-        <v>390</v>
+        <v>441</v>
       </c>
       <c r="R6" t="s">
-        <v>391</v>
+        <v>442</v>
       </c>
       <c r="S6" t="s">
-        <v>392</v>
+        <v>443</v>
       </c>
       <c r="T6" t="s">
-        <v>393</v>
+        <v>444</v>
       </c>
       <c r="U6" t="s">
-        <v>394</v>
+        <v>445</v>
       </c>
       <c r="V6" t="s">
-        <v>395</v>
+        <v>446</v>
       </c>
       <c r="W6" t="s">
-        <v>396</v>
+        <v>447</v>
       </c>
       <c r="X6" t="s">
-        <v>397</v>
+        <v>448</v>
       </c>
       <c r="Y6" t="s">
-        <v>398</v>
+        <v>449</v>
       </c>
       <c r="Z6" t="s">
-        <v>399</v>
+        <v>450</v>
       </c>
       <c r="AA6" t="s">
-        <v>400</v>
+        <v>451</v>
       </c>
       <c r="AB6" t="n">
         <v>2</v>
@@ -3489,93 +4275,93 @@
         <v>1</v>
       </c>
       <c r="AD6" t="s">
-        <v>401</v>
+        <v>452</v>
       </c>
       <c r="AE6" t="s">
-        <v>402</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>403</v>
+        <v>454</v>
       </c>
       <c r="B7" t="s">
-        <v>404</v>
+        <v>455</v>
       </c>
       <c r="C7" t="s">
-        <v>405</v>
+        <v>456</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>406</v>
+        <v>457</v>
       </c>
       <c r="F7" t="s">
-        <v>407</v>
+        <v>458</v>
       </c>
       <c r="G7" t="s">
-        <v>408</v>
+        <v>459</v>
       </c>
       <c r="H7" t="s">
-        <v>409</v>
+        <v>460</v>
       </c>
       <c r="I7" t="s">
-        <v>410</v>
+        <v>461</v>
       </c>
       <c r="J7" t="s">
-        <v>411</v>
+        <v>462</v>
       </c>
       <c r="K7" t="s">
-        <v>412</v>
+        <v>463</v>
       </c>
       <c r="L7" t="s">
-        <v>413</v>
+        <v>464</v>
       </c>
       <c r="M7" t="s">
-        <v>414</v>
+        <v>465</v>
       </c>
       <c r="N7" t="s">
-        <v>415</v>
+        <v>466</v>
       </c>
       <c r="O7" t="s">
-        <v>416</v>
+        <v>467</v>
       </c>
       <c r="P7" t="s">
-        <v>417</v>
+        <v>468</v>
       </c>
       <c r="Q7" t="s">
-        <v>418</v>
+        <v>469</v>
       </c>
       <c r="R7" t="s">
-        <v>419</v>
+        <v>470</v>
       </c>
       <c r="S7" t="s">
-        <v>420</v>
+        <v>471</v>
       </c>
       <c r="T7" t="s">
-        <v>421</v>
+        <v>472</v>
       </c>
       <c r="U7" t="s">
-        <v>422</v>
+        <v>473</v>
       </c>
       <c r="V7" t="s">
-        <v>423</v>
+        <v>474</v>
       </c>
       <c r="W7" t="s">
-        <v>424</v>
+        <v>475</v>
       </c>
       <c r="X7" t="s">
-        <v>425</v>
+        <v>476</v>
       </c>
       <c r="Y7" t="s">
-        <v>426</v>
+        <v>477</v>
       </c>
       <c r="Z7" t="s">
-        <v>427</v>
+        <v>478</v>
       </c>
       <c r="AA7" t="s">
-        <v>428</v>
+        <v>479</v>
       </c>
       <c r="AB7" t="n">
         <v>2</v>
@@ -3584,89 +4370,89 @@
         <v>1</v>
       </c>
       <c r="AD7" t="s">
-        <v>429</v>
+        <v>480</v>
       </c>
       <c r="AE7" t="s">
-        <v>430</v>
+        <v>481</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>431</v>
+        <v>482</v>
       </c>
       <c r="B8" t="s">
-        <v>432</v>
+        <v>483</v>
       </c>
       <c r="C8" t="s">
-        <v>433</v>
+        <v>484</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>434</v>
+        <v>485</v>
       </c>
       <c r="F8" t="s">
-        <v>435</v>
+        <v>486</v>
       </c>
       <c r="G8" t="s">
-        <v>436</v>
+        <v>487</v>
       </c>
       <c r="H8" t="s">
-        <v>437</v>
+        <v>488</v>
       </c>
       <c r="I8" t="s">
-        <v>438</v>
+        <v>489</v>
       </c>
       <c r="J8"/>
       <c r="K8" t="s">
-        <v>439</v>
+        <v>490</v>
       </c>
       <c r="L8" t="s">
-        <v>440</v>
+        <v>491</v>
       </c>
       <c r="M8" t="s">
-        <v>441</v>
+        <v>492</v>
       </c>
       <c r="N8" t="s">
-        <v>442</v>
+        <v>493</v>
       </c>
       <c r="O8" t="s">
-        <v>443</v>
+        <v>494</v>
       </c>
       <c r="P8" t="s">
-        <v>444</v>
+        <v>495</v>
       </c>
       <c r="Q8" t="s">
-        <v>445</v>
+        <v>496</v>
       </c>
       <c r="R8"/>
       <c r="S8" t="s">
-        <v>446</v>
+        <v>497</v>
       </c>
       <c r="T8" t="s">
-        <v>447</v>
+        <v>498</v>
       </c>
       <c r="U8" t="s">
-        <v>448</v>
+        <v>499</v>
       </c>
       <c r="V8" t="s">
-        <v>449</v>
+        <v>500</v>
       </c>
       <c r="W8" t="s">
-        <v>450</v>
+        <v>501</v>
       </c>
       <c r="X8" t="s">
-        <v>451</v>
+        <v>502</v>
       </c>
       <c r="Y8" t="s">
-        <v>452</v>
+        <v>503</v>
       </c>
       <c r="Z8" t="s">
-        <v>453</v>
+        <v>504</v>
       </c>
       <c r="AA8" t="s">
-        <v>454</v>
+        <v>505</v>
       </c>
       <c r="AB8" t="n">
         <v>2</v>
@@ -3675,93 +4461,93 @@
         <v>1</v>
       </c>
       <c r="AD8" t="s">
-        <v>455</v>
+        <v>506</v>
       </c>
       <c r="AE8" t="s">
-        <v>456</v>
+        <v>507</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>457</v>
+        <v>508</v>
       </c>
       <c r="B9" t="s">
-        <v>458</v>
+        <v>509</v>
       </c>
       <c r="C9" t="s">
-        <v>459</v>
+        <v>510</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>460</v>
+        <v>511</v>
       </c>
       <c r="F9" t="s">
-        <v>461</v>
+        <v>512</v>
       </c>
       <c r="G9" t="s">
-        <v>462</v>
+        <v>513</v>
       </c>
       <c r="H9" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="I9" t="s">
-        <v>464</v>
+        <v>515</v>
       </c>
       <c r="J9" t="s">
-        <v>465</v>
+        <v>516</v>
       </c>
       <c r="K9" t="s">
-        <v>466</v>
+        <v>517</v>
       </c>
       <c r="L9" t="s">
-        <v>467</v>
+        <v>518</v>
       </c>
       <c r="M9" t="s">
-        <v>468</v>
+        <v>519</v>
       </c>
       <c r="N9" t="s">
-        <v>469</v>
+        <v>520</v>
       </c>
       <c r="O9" t="s">
-        <v>470</v>
+        <v>521</v>
       </c>
       <c r="P9" t="s">
-        <v>471</v>
+        <v>522</v>
       </c>
       <c r="Q9" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="R9" t="s">
-        <v>473</v>
+        <v>524</v>
       </c>
       <c r="S9" t="s">
-        <v>474</v>
+        <v>525</v>
       </c>
       <c r="T9" t="s">
-        <v>475</v>
+        <v>526</v>
       </c>
       <c r="U9" t="s">
-        <v>476</v>
+        <v>527</v>
       </c>
       <c r="V9" t="s">
-        <v>477</v>
+        <v>528</v>
       </c>
       <c r="W9" t="s">
-        <v>478</v>
+        <v>529</v>
       </c>
       <c r="X9" t="s">
-        <v>479</v>
+        <v>530</v>
       </c>
       <c r="Y9" t="s">
-        <v>480</v>
+        <v>531</v>
       </c>
       <c r="Z9" t="s">
-        <v>481</v>
+        <v>532</v>
       </c>
       <c r="AA9" t="s">
-        <v>482</v>
+        <v>533</v>
       </c>
       <c r="AB9" t="n">
         <v>2</v>
@@ -3770,10 +4556,10 @@
         <v>1</v>
       </c>
       <c r="AD9" t="s">
-        <v>483</v>
+        <v>534</v>
       </c>
       <c r="AE9" t="s">
-        <v>484</v>
+        <v>535</v>
       </c>
     </row>
   </sheetData>
@@ -3785,547 +4571,547 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>485</v>
+        <v>536</v>
       </c>
       <c r="B1" t="s">
-        <v>486</v>
+        <v>537</v>
       </c>
       <c r="C1" t="s">
-        <v>487</v>
+        <v>538</v>
       </c>
       <c r="D1" t="s">
-        <v>488</v>
+        <v>539</v>
       </c>
       <c r="E1" t="s">
-        <v>489</v>
+        <v>540</v>
       </c>
       <c r="F1" t="s">
-        <v>490</v>
+        <v>541</v>
       </c>
       <c r="G1" t="s">
-        <v>491</v>
+        <v>542</v>
       </c>
       <c r="H1" t="s">
-        <v>492</v>
+        <v>543</v>
       </c>
       <c r="I1" t="s">
-        <v>493</v>
+        <v>544</v>
       </c>
       <c r="J1" t="s">
-        <v>494</v>
+        <v>545</v>
       </c>
       <c r="K1" t="s">
-        <v>495</v>
+        <v>546</v>
       </c>
       <c r="L1" t="s">
-        <v>496</v>
+        <v>547</v>
       </c>
       <c r="M1" t="s">
-        <v>497</v>
+        <v>548</v>
       </c>
       <c r="N1" t="s">
-        <v>498</v>
+        <v>549</v>
       </c>
       <c r="O1" t="s">
-        <v>499</v>
+        <v>550</v>
       </c>
       <c r="P1" t="s">
-        <v>500</v>
+        <v>551</v>
       </c>
       <c r="Q1" t="s">
-        <v>501</v>
+        <v>552</v>
       </c>
       <c r="R1" t="s">
-        <v>502</v>
+        <v>553</v>
       </c>
       <c r="S1" t="s">
-        <v>503</v>
+        <v>554</v>
       </c>
       <c r="T1" t="s">
-        <v>504</v>
+        <v>555</v>
       </c>
       <c r="U1" t="s">
-        <v>505</v>
+        <v>556</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>506</v>
+        <v>557</v>
       </c>
       <c r="B2" t="s">
-        <v>507</v>
+        <v>558</v>
       </c>
       <c r="C2" t="s">
-        <v>508</v>
+        <v>559</v>
       </c>
       <c r="D2" t="s">
-        <v>509</v>
+        <v>560</v>
       </c>
       <c r="E2" t="s">
-        <v>510</v>
+        <v>561</v>
       </c>
       <c r="F2" t="s">
-        <v>511</v>
+        <v>562</v>
       </c>
       <c r="G2" t="s">
-        <v>512</v>
+        <v>563</v>
       </c>
       <c r="H2" t="s">
-        <v>513</v>
+        <v>564</v>
       </c>
       <c r="I2" t="s">
-        <v>514</v>
+        <v>565</v>
       </c>
       <c r="J2" t="s">
-        <v>515</v>
+        <v>566</v>
       </c>
       <c r="K2"/>
       <c r="L2" t="n">
         <v>82</v>
       </c>
       <c r="M2" t="s">
-        <v>516</v>
+        <v>567</v>
       </c>
       <c r="N2" t="s">
-        <v>517</v>
+        <v>568</v>
       </c>
       <c r="O2" t="s">
-        <v>518</v>
+        <v>569</v>
       </c>
       <c r="P2" t="s">
-        <v>519</v>
+        <v>570</v>
       </c>
       <c r="Q2" t="s">
-        <v>520</v>
+        <v>571</v>
       </c>
       <c r="R2" t="s">
-        <v>521</v>
+        <v>572</v>
       </c>
       <c r="S2" t="s">
-        <v>522</v>
+        <v>573</v>
       </c>
       <c r="T2" t="s">
-        <v>523</v>
+        <v>574</v>
       </c>
       <c r="U2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>524</v>
+        <v>575</v>
       </c>
       <c r="B3" t="s">
-        <v>525</v>
+        <v>576</v>
       </c>
       <c r="C3" t="s">
-        <v>526</v>
+        <v>577</v>
       </c>
       <c r="D3" t="s">
-        <v>527</v>
+        <v>578</v>
       </c>
       <c r="E3" t="s">
-        <v>528</v>
+        <v>579</v>
       </c>
       <c r="F3" t="s">
-        <v>529</v>
+        <v>580</v>
       </c>
       <c r="G3" t="s">
-        <v>530</v>
+        <v>581</v>
       </c>
       <c r="H3" t="s">
-        <v>531</v>
+        <v>582</v>
       </c>
       <c r="I3" t="s">
-        <v>532</v>
+        <v>583</v>
       </c>
       <c r="J3" t="s">
-        <v>533</v>
+        <v>584</v>
       </c>
       <c r="K3"/>
       <c r="L3" t="n">
         <v>91</v>
       </c>
       <c r="M3" t="s">
-        <v>534</v>
+        <v>585</v>
       </c>
       <c r="N3" t="s">
-        <v>535</v>
+        <v>586</v>
       </c>
       <c r="O3"/>
       <c r="P3" t="s">
-        <v>536</v>
+        <v>587</v>
       </c>
       <c r="Q3" t="s">
-        <v>537</v>
+        <v>588</v>
       </c>
       <c r="R3" t="s">
-        <v>538</v>
+        <v>589</v>
       </c>
       <c r="S3" t="s">
-        <v>539</v>
+        <v>590</v>
       </c>
       <c r="T3" t="s">
-        <v>540</v>
+        <v>591</v>
       </c>
       <c r="U3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>541</v>
+        <v>592</v>
       </c>
       <c r="B4" t="s">
-        <v>542</v>
+        <v>593</v>
       </c>
       <c r="C4" t="s">
-        <v>543</v>
+        <v>594</v>
       </c>
       <c r="D4" t="s">
-        <v>544</v>
+        <v>595</v>
       </c>
       <c r="E4" t="s">
-        <v>545</v>
+        <v>596</v>
       </c>
       <c r="F4" t="s">
-        <v>546</v>
+        <v>597</v>
       </c>
       <c r="G4" t="s">
-        <v>547</v>
+        <v>598</v>
       </c>
       <c r="H4" t="s">
-        <v>548</v>
+        <v>599</v>
       </c>
       <c r="I4" t="s">
-        <v>549</v>
+        <v>600</v>
       </c>
       <c r="J4" t="s">
-        <v>550</v>
+        <v>601</v>
       </c>
       <c r="K4"/>
       <c r="L4" t="n">
         <v>74</v>
       </c>
       <c r="M4" t="s">
-        <v>551</v>
+        <v>602</v>
       </c>
       <c r="N4" t="s">
-        <v>552</v>
+        <v>603</v>
       </c>
       <c r="O4" t="s">
-        <v>553</v>
+        <v>604</v>
       </c>
       <c r="P4" t="s">
-        <v>554</v>
+        <v>605</v>
       </c>
       <c r="Q4" t="s">
-        <v>555</v>
+        <v>606</v>
       </c>
       <c r="R4" t="s">
-        <v>556</v>
+        <v>607</v>
       </c>
       <c r="S4" t="s">
-        <v>557</v>
+        <v>608</v>
       </c>
       <c r="T4" t="s">
-        <v>558</v>
+        <v>609</v>
       </c>
       <c r="U4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>559</v>
+        <v>610</v>
       </c>
       <c r="B5" t="s">
-        <v>560</v>
+        <v>611</v>
       </c>
       <c r="C5" t="s">
-        <v>561</v>
+        <v>612</v>
       </c>
       <c r="D5" t="s">
-        <v>562</v>
+        <v>613</v>
       </c>
       <c r="E5" t="s">
-        <v>563</v>
+        <v>614</v>
       </c>
       <c r="F5" t="s">
-        <v>564</v>
+        <v>615</v>
       </c>
       <c r="G5" t="s">
-        <v>565</v>
+        <v>616</v>
       </c>
       <c r="H5" t="s">
-        <v>566</v>
+        <v>617</v>
       </c>
       <c r="I5" t="s">
-        <v>567</v>
+        <v>618</v>
       </c>
       <c r="J5" t="s">
-        <v>568</v>
+        <v>619</v>
       </c>
       <c r="K5"/>
       <c r="L5" t="n">
         <v>88</v>
       </c>
       <c r="M5" t="s">
-        <v>569</v>
+        <v>620</v>
       </c>
       <c r="N5" t="s">
-        <v>570</v>
+        <v>621</v>
       </c>
       <c r="O5" t="s">
-        <v>571</v>
+        <v>622</v>
       </c>
       <c r="P5" t="s">
-        <v>572</v>
+        <v>623</v>
       </c>
       <c r="Q5" t="s">
-        <v>573</v>
+        <v>624</v>
       </c>
       <c r="R5" t="s">
-        <v>574</v>
+        <v>625</v>
       </c>
       <c r="S5" t="s">
-        <v>575</v>
+        <v>626</v>
       </c>
       <c r="T5" t="s">
-        <v>576</v>
+        <v>627</v>
       </c>
       <c r="U5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>577</v>
+        <v>628</v>
       </c>
       <c r="B6" t="s">
-        <v>578</v>
+        <v>629</v>
       </c>
       <c r="C6" t="s">
-        <v>579</v>
+        <v>630</v>
       </c>
       <c r="D6" t="s">
-        <v>580</v>
+        <v>631</v>
       </c>
       <c r="E6" t="s">
-        <v>581</v>
+        <v>632</v>
       </c>
       <c r="F6" t="s">
-        <v>582</v>
+        <v>633</v>
       </c>
       <c r="G6" t="s">
-        <v>583</v>
+        <v>634</v>
       </c>
       <c r="H6" t="s">
-        <v>584</v>
+        <v>635</v>
       </c>
       <c r="I6" t="s">
-        <v>585</v>
+        <v>636</v>
       </c>
       <c r="J6" t="s">
-        <v>586</v>
+        <v>637</v>
       </c>
       <c r="K6"/>
       <c r="L6" t="n">
         <v>76</v>
       </c>
       <c r="M6" t="s">
-        <v>587</v>
+        <v>638</v>
       </c>
       <c r="N6" t="s">
-        <v>588</v>
+        <v>639</v>
       </c>
       <c r="O6"/>
       <c r="P6" t="s">
-        <v>589</v>
+        <v>640</v>
       </c>
       <c r="Q6" t="s">
-        <v>590</v>
+        <v>641</v>
       </c>
       <c r="R6" t="s">
-        <v>591</v>
+        <v>642</v>
       </c>
       <c r="S6" t="s">
-        <v>592</v>
+        <v>643</v>
       </c>
       <c r="T6" t="s">
-        <v>593</v>
+        <v>644</v>
       </c>
       <c r="U6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>594</v>
+        <v>645</v>
       </c>
       <c r="B7" t="s">
-        <v>595</v>
+        <v>646</v>
       </c>
       <c r="C7" t="s">
-        <v>596</v>
+        <v>647</v>
       </c>
       <c r="D7" t="s">
-        <v>597</v>
+        <v>648</v>
       </c>
       <c r="E7" t="s">
-        <v>598</v>
+        <v>649</v>
       </c>
       <c r="F7" t="s">
-        <v>599</v>
+        <v>650</v>
       </c>
       <c r="G7" t="s">
-        <v>600</v>
+        <v>651</v>
       </c>
       <c r="H7" t="s">
-        <v>601</v>
+        <v>652</v>
       </c>
       <c r="I7" t="s">
-        <v>602</v>
+        <v>653</v>
       </c>
       <c r="J7" t="s">
-        <v>603</v>
+        <v>654</v>
       </c>
       <c r="K7"/>
       <c r="L7" t="n">
         <v>93</v>
       </c>
       <c r="M7" t="s">
-        <v>604</v>
+        <v>655</v>
       </c>
       <c r="N7" t="s">
-        <v>605</v>
+        <v>656</v>
       </c>
       <c r="O7"/>
       <c r="P7" t="s">
-        <v>606</v>
+        <v>657</v>
       </c>
       <c r="Q7" t="s">
-        <v>607</v>
+        <v>658</v>
       </c>
       <c r="R7" t="s">
-        <v>608</v>
+        <v>659</v>
       </c>
       <c r="S7" t="s">
-        <v>609</v>
+        <v>660</v>
       </c>
       <c r="T7" t="s">
-        <v>610</v>
+        <v>661</v>
       </c>
       <c r="U7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>611</v>
+        <v>662</v>
       </c>
       <c r="B8" t="s">
-        <v>612</v>
+        <v>663</v>
       </c>
       <c r="C8" t="s">
-        <v>613</v>
+        <v>664</v>
       </c>
       <c r="D8" t="s">
-        <v>614</v>
+        <v>665</v>
       </c>
       <c r="E8" t="s">
-        <v>615</v>
+        <v>666</v>
       </c>
       <c r="F8" t="s">
-        <v>616</v>
+        <v>667</v>
       </c>
       <c r="G8" t="s">
-        <v>617</v>
+        <v>668</v>
       </c>
       <c r="H8" t="s">
-        <v>618</v>
+        <v>669</v>
       </c>
       <c r="I8" t="s">
-        <v>619</v>
+        <v>670</v>
       </c>
       <c r="J8" t="s">
-        <v>620</v>
+        <v>671</v>
       </c>
       <c r="K8"/>
       <c r="L8" t="n">
         <v>71</v>
       </c>
       <c r="M8" t="s">
-        <v>621</v>
+        <v>672</v>
       </c>
       <c r="N8" t="s">
-        <v>622</v>
+        <v>673</v>
       </c>
       <c r="O8"/>
       <c r="P8" t="s">
-        <v>623</v>
+        <v>674</v>
       </c>
       <c r="Q8" t="s">
-        <v>624</v>
+        <v>675</v>
       </c>
       <c r="R8" t="s">
-        <v>625</v>
+        <v>676</v>
       </c>
       <c r="S8" t="s">
-        <v>626</v>
+        <v>677</v>
       </c>
       <c r="T8" t="s">
-        <v>627</v>
+        <v>678</v>
       </c>
       <c r="U8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>628</v>
+        <v>679</v>
       </c>
       <c r="B9" t="s">
-        <v>629</v>
+        <v>680</v>
       </c>
       <c r="C9" t="s">
-        <v>630</v>
+        <v>681</v>
       </c>
       <c r="D9" t="s">
-        <v>631</v>
+        <v>682</v>
       </c>
       <c r="E9" t="s">
-        <v>632</v>
+        <v>683</v>
       </c>
       <c r="F9" t="s">
-        <v>633</v>
+        <v>684</v>
       </c>
       <c r="G9" t="s">
-        <v>634</v>
+        <v>685</v>
       </c>
       <c r="H9" t="s">
-        <v>635</v>
+        <v>686</v>
       </c>
       <c r="I9" t="s">
-        <v>636</v>
+        <v>687</v>
       </c>
       <c r="J9" t="s">
-        <v>637</v>
+        <v>688</v>
       </c>
       <c r="K9"/>
       <c r="L9" t="n">
         <v>85</v>
       </c>
       <c r="M9" t="s">
-        <v>638</v>
+        <v>689</v>
       </c>
       <c r="N9" t="s">
-        <v>639</v>
+        <v>690</v>
       </c>
       <c r="O9"/>
       <c r="P9" t="s">
-        <v>640</v>
+        <v>691</v>
       </c>
       <c r="Q9" t="s">
-        <v>641</v>
+        <v>692</v>
       </c>
       <c r="R9" t="s">
-        <v>642</v>
+        <v>693</v>
       </c>
       <c r="S9" t="s">
-        <v>643</v>
+        <v>694</v>
       </c>
       <c r="T9" t="s">
-        <v>644</v>
+        <v>695</v>
       </c>
       <c r="U9" t="s">
-        <v>645</v>
+        <v>696</v>
       </c>
     </row>
   </sheetData>
@@ -4337,12 +5123,1302 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>646</v>
+        <v>697</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>647</v>
+        <v>698</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+    </row>
+    <row r="4">
+      <c r="A4"/>
+    </row>
+    <row r="5">
+      <c r="A5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>701</v>
+      </c>
+      <c r="B6" t="s">
+        <v>702</v>
+      </c>
+      <c r="C6" t="s">
+        <v>703</v>
+      </c>
+      <c r="D6" t="s">
+        <v>704</v>
+      </c>
+      <c r="E6" t="s">
+        <v>705</v>
+      </c>
+      <c r="F6" t="s">
+        <v>706</v>
+      </c>
+      <c r="G6" t="s">
+        <v>707</v>
+      </c>
+      <c r="H6" t="s">
+        <v>708</v>
+      </c>
+      <c r="I6" t="s">
+        <v>709</v>
+      </c>
+      <c r="J6" t="s">
+        <v>710</v>
+      </c>
+      <c r="K6" t="s">
+        <v>711</v>
+      </c>
+      <c r="L6" t="s">
+        <v>712</v>
+      </c>
+      <c r="M6" t="s">
+        <v>713</v>
+      </c>
+      <c r="N6" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>715</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="C7" t="s">
+        <v>716</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>717</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>718</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>719</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>720</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8" t="n">
+        <v>-2.0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1.82</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>721</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>722</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="s">
+        <v>723</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>724</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>725</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>726</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10"/>
+      <c r="K10"/>
+      <c r="L10"/>
+      <c r="M10"/>
+      <c r="N10" t="n">
+        <v>-2.73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>727</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>728</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>729</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="N11" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>730</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>731</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>732</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12"/>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>733</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C13" t="s">
+        <v>734</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>735</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>736</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>737</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>738</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14"/>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14"/>
+      <c r="N14" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>739</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>740</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>741</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15"/>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15"/>
+      <c r="N15" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>742</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C16" t="s">
+        <v>743</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
+        <v>744</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16"/>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16"/>
+      <c r="N16" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>745</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>746</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>747</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17"/>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>748</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>749</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
+        <v>750</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>751</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>752</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>753</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19"/>
+      <c r="K19"/>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>754</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>755</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="s">
+        <v>756</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>757</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>758</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>759</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+      <c r="N21" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>760</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C22" t="s">
+        <v>761</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="s">
+        <v>762</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22"/>
+      <c r="K22"/>
+      <c r="L22"/>
+      <c r="M22"/>
+      <c r="N22" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>763</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C23" t="s">
+        <v>764</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>765</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>766</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C24" t="s">
+        <v>767</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="s">
+        <v>768</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>769</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C25" t="s">
+        <v>770</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>771</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25"/>
+      <c r="K25"/>
+      <c r="L25"/>
+      <c r="M25"/>
+      <c r="N25" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>772</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>773</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>774</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26"/>
+      <c r="K26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+      <c r="N26" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>775</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>776</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>777</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27"/>
+      <c r="K27"/>
+      <c r="L27"/>
+      <c r="M27" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>778</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>779</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="s">
+        <v>780</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>781</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>782</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="s">
+        <v>783</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29"/>
+      <c r="K29"/>
+      <c r="L29"/>
+      <c r="M29"/>
+      <c r="N29" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>784</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C30" t="s">
+        <v>785</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="s">
+        <v>786</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30"/>
+      <c r="K30"/>
+      <c r="L30"/>
+      <c r="M30"/>
+      <c r="N30" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>787</v>
+      </c>
+      <c r="B32" t="s">
+        <v>788</v>
+      </c>
+      <c r="C32" t="s">
+        <v>789</v>
+      </c>
+      <c r="D32" t="s">
+        <v>790</v>
+      </c>
+      <c r="E32" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>792</v>
+      </c>
+      <c r="B33" t="s">
+        <v>793</v>
+      </c>
+      <c r="C33" t="s">
+        <v>794</v>
+      </c>
+      <c r="D33" t="s">
+        <v>795</v>
+      </c>
+      <c r="E33" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>797</v>
+      </c>
+      <c r="B34" t="s">
+        <v>798</v>
+      </c>
+      <c r="C34" t="s">
+        <v>799</v>
+      </c>
+      <c r="D34" t="s">
+        <v>800</v>
+      </c>
+      <c r="E34" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>803</v>
+      </c>
+      <c r="B37" t="s">
+        <v>804</v>
+      </c>
+      <c r="C37" t="s">
+        <v>805</v>
+      </c>
+      <c r="D37" t="s">
+        <v>806</v>
+      </c>
+      <c r="E37" t="s">
+        <v>807</v>
+      </c>
+      <c r="F37" t="s">
+        <v>808</v>
+      </c>
+      <c r="G37" t="s">
+        <v>809</v>
+      </c>
+      <c r="H37" t="s">
+        <v>810</v>
+      </c>
+      <c r="I37" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>812</v>
+      </c>
+      <c r="B38" t="s">
+        <v>813</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="s">
+        <v>814</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="s">
+        <v>815</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>816</v>
+      </c>
+      <c r="B39" t="s">
+        <v>817</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="s">
+        <v>818</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="s">
+        <v>819</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.82</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>820</v>
+      </c>
+      <c r="B40" t="s">
+        <v>821</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="s">
+        <v>822</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="s">
+        <v>823</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>824</v>
+      </c>
+      <c r="B41" t="s">
+        <v>825</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>826</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="s">
+        <v>827</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-0.7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>828</v>
+      </c>
+      <c r="B42" t="s">
+        <v>829</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>830</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="s">
+        <v>831</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>832</v>
+      </c>
+      <c r="B43" t="s">
+        <v>833</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="s">
+        <v>834</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="s">
+        <v>835</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>836</v>
+      </c>
+      <c r="B44" t="s">
+        <v>837</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="s">
+        <v>838</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="s">
+        <v>839</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>840</v>
+      </c>
+      <c r="B45" t="s">
+        <v>841</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="s">
+        <v>842</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="s">
+        <v>843</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>844</v>
+      </c>
+      <c r="B46" t="s">
+        <v>845</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="s">
+        <v>846</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="s">
+        <v>847</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Record Splits to the members-only /bets board. (#227)
sj bets now reads the Record Splits sheet by header names (Bettor, Source
tab, Class, Sport) instead of fixed ranges, writes record_splits.json, and
tolerates the new Bets Pick Class column. Lockedin_Sportz (Z-) is mapped
like LC; any P/L for him is labeled hypothetical 1u because he posts no
stake or units. The portal adds a Record splits tab with fade highlighting.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Austin Wiley <thejayer@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/bets/tracker_tabs.xlsx
+++ b/tests/fixtures/bets/tracker_tabs.xlsx
@@ -6,12 +6,13 @@
     <sheet name="Parlay Legs" sheetId="2" r:id="rId2"/>
     <sheet name="BetMGM Public Warnings" sheetId="3" r:id="rId3"/>
     <sheet name="Summary" sheetId="4" r:id="rId4"/>
+    <sheet name="Record Splits" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="848">
   <si>
     <t>Bet ID</t>
   </si>
@@ -103,6 +104,9 @@
     <t>Settled units (helper)</t>
   </si>
   <si>
+    <t>Pick Class</t>
+  </si>
+  <si>
     <t>Extra unused</t>
   </si>
   <si>
@@ -166,6 +170,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -226,6 +233,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -286,6 +296,9 @@
     <t>Parlay/multi-leg</t>
   </si>
   <si>
+    <t>Parlay</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -349,6 +362,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -409,6 +425,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -469,6 +488,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -529,6 +551,9 @@
     <t>Parlay/multi-leg</t>
   </si>
   <si>
+    <t>Parlay</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -592,6 +617,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Prop</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -652,6 +680,9 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
@@ -715,9 +746,132 @@
     <t>Single</t>
   </si>
   <si>
+    <t>Team</t>
+  </si>
+  <si>
     <t>ignore-me</t>
   </si>
   <si>
+    <t>Z-1</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>2026-09-18 12:00:00</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>8:20 PM</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>player prop</t>
+  </si>
+  <si>
+    <t>Mahomes over 249.5 pass yds</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>graded</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>https://x.com/Lockedin_Sportz/status/1</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>ignore-me</t>
+  </si>
+  <si>
+    <t>Z-2</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>2026-09-18 12:00:00</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>Thursday</t>
+  </si>
+  <si>
+    <t>8:20 PM</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>player prop</t>
+  </si>
+  <si>
+    <t>Kelce over 59.5 rec yds</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>graded</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>https://x.com/Lockedin_Sportz/status/1</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>ignore-me</t>
+  </si>
+  <si>
     <t>Leg ID</t>
   </si>
   <si>
@@ -1955,6 +2109,453 @@
   </si>
   <si>
     <t>do not read</t>
+  </si>
+  <si>
+    <t>Record Splits</t>
+  </si>
+  <si>
+    <t>Synthetic fixture — not live data</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Win %</t>
+  </si>
+  <si>
+    <t>Bettor</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Source tab</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Posted units P&amp;L</t>
+  </si>
+  <si>
+    <t>$ P&amp;L</t>
+  </si>
+  <si>
+    <t>$ staked</t>
+  </si>
+  <si>
+    <t>Flat 1u</t>
+  </si>
+  <si>
+    <t>1u fade at -110</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>Steve</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>chellgod</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>chellgod</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>chellgod</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>btidy216</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>btidy216</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>btidy216</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Team pick</t>
+  </si>
+  <si>
+    <t>@Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Player prop</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Parlay Legs</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Expected</t>
+  </si>
+  <si>
+    <t>Actual</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Bets W vs splits</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Parlay legs vs splits</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Sport split</t>
+  </si>
+  <si>
+    <t>Sport</t>
+  </si>
+  <si>
+    <t>Bettor</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>Source tab</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Win %</t>
+  </si>
+  <si>
+    <t>1u fade at -110</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>CFB</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>MLB</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Parlay</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>Lockedin_Sportz</t>
+  </si>
+  <si>
+    <t>Prop</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>NFL</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
+  </si>
+  <si>
+    <t>CFB</t>
+  </si>
+  <si>
+    <t>Trent</t>
+  </si>
+  <si>
+    <t>Team</t>
+  </si>
+  <si>
+    <t>Bets</t>
   </si>
 </sst>
 </file>
@@ -2081,55 +2682,58 @@
       <c r="AE1" t="s">
         <v>30</v>
       </c>
+      <c r="AF1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N2" t="n">
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="P2" t="n">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="Q2" t="n">
         <v>100</v>
@@ -2139,77 +2743,80 @@
         <v>100</v>
       </c>
       <c r="T2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="U2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="V2"/>
       <c r="W2"/>
       <c r="X2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Y2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="Z2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AA2"/>
       <c r="AB2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="AC2" t="n">
         <v>100</v>
       </c>
       <c r="AD2"/>
       <c r="AE2" t="s">
-        <v>51</v>
+        <v>52</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I3"/>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="N3" t="n">
         <v>1</v>
       </c>
       <c r="O3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="P3" t="n">
         <v>1.909</v>
@@ -2224,25 +2831,25 @@
         <v>100</v>
       </c>
       <c r="T3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="U3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="V3"/>
       <c r="W3"/>
       <c r="X3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="Y3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="Z3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="AA3"/>
       <c r="AB3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="AC3" t="n">
         <v>110</v>
@@ -2251,55 +2858,58 @@
         <v>1</v>
       </c>
       <c r="AE3" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="D4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="I4"/>
       <c r="J4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="L4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="M4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="N4" t="n">
         <v>2</v>
       </c>
       <c r="O4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="P4" t="n">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="Q4" t="n">
         <v>50</v>
@@ -2309,79 +2919,82 @@
         <v>150</v>
       </c>
       <c r="T4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="U4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="V4"/>
       <c r="W4"/>
       <c r="X4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="Y4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="Z4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="AA4"/>
       <c r="AB4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="AC4" t="n">
         <v>50</v>
       </c>
       <c r="AD4"/>
       <c r="AE4" t="s">
-        <v>91</v>
+        <v>94</v>
+      </c>
+      <c r="AF4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="G5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="I5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="J5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="K5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="M5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
       </c>
       <c r="O5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="P5" t="n">
         <v>2.5</v>
@@ -2394,77 +3007,80 @@
         <v>2500</v>
       </c>
       <c r="T5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="U5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="V5"/>
       <c r="W5"/>
       <c r="X5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="Y5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="Z5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="AA5"/>
       <c r="AB5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="AC5" t="n">
         <v>1000</v>
       </c>
       <c r="AD5"/>
       <c r="AE5" t="s">
-        <v>112</v>
+        <v>116</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B6" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="E6" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F6" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="G6" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="I6"/>
       <c r="J6" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="K6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="L6" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="M6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="N6" t="n">
         <v>1</v>
       </c>
       <c r="O6" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="P6" t="n">
         <v>1.909</v>
@@ -2477,77 +3093,80 @@
         <v>1818</v>
       </c>
       <c r="T6" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="U6" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="V6"/>
       <c r="W6"/>
       <c r="X6" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="Y6" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="Z6" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="AA6"/>
       <c r="AB6" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="AC6" t="n">
         <v>2000</v>
       </c>
       <c r="AD6"/>
       <c r="AE6" t="s">
-        <v>132</v>
+        <v>137</v>
+      </c>
+      <c r="AF6" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C7" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E7" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="F7" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="G7" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="H7" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="I7"/>
       <c r="J7" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="K7" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="L7" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="M7" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="N7" t="n">
         <v>1</v>
       </c>
       <c r="O7" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="P7" t="n">
         <v>1.5</v>
@@ -2560,77 +3179,80 @@
         <v>200</v>
       </c>
       <c r="T7" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="U7" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="V7"/>
       <c r="W7"/>
       <c r="X7" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="Y7" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="Z7" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="AA7"/>
       <c r="AB7" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="AC7" t="n">
         <v>400</v>
       </c>
       <c r="AD7"/>
       <c r="AE7" t="s">
-        <v>152</v>
+        <v>158</v>
+      </c>
+      <c r="AF7" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B8" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C8" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D8" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="E8" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="F8" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="G8" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="H8" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="I8"/>
       <c r="J8" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="K8" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="L8" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="M8" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="N8" t="n">
         <v>2</v>
       </c>
       <c r="O8" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="P8" t="n">
         <v>3.5</v>
@@ -2643,79 +3265,82 @@
         <v>100</v>
       </c>
       <c r="T8" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="U8" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="V8"/>
       <c r="W8"/>
       <c r="X8" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="Y8" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="Z8" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="AA8"/>
       <c r="AB8" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="AC8" t="n">
         <v>40</v>
       </c>
       <c r="AD8"/>
       <c r="AE8" t="s">
-        <v>172</v>
+        <v>179</v>
+      </c>
+      <c r="AF8" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B9" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="C9" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D9" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="E9" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="F9" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="G9" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="H9" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="I9" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="J9" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="K9" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="L9" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="M9" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="N9" t="n">
         <v>1</v>
       </c>
       <c r="O9" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="P9" t="n">
         <v>1.833</v>
@@ -2728,77 +3353,80 @@
         <v>50</v>
       </c>
       <c r="T9" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="U9" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="V9"/>
       <c r="W9"/>
       <c r="X9" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="Y9" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="Z9" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="AA9"/>
       <c r="AB9" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="AC9" t="n">
         <v>60</v>
       </c>
       <c r="AD9"/>
       <c r="AE9" t="s">
-        <v>193</v>
+        <v>201</v>
+      </c>
+      <c r="AF9" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>194</v>
+        <v>203</v>
       </c>
       <c r="B10" t="s">
-        <v>195</v>
+        <v>204</v>
       </c>
       <c r="C10" t="s">
-        <v>196</v>
+        <v>205</v>
       </c>
       <c r="D10" t="s">
-        <v>197</v>
+        <v>206</v>
       </c>
       <c r="E10" t="s">
-        <v>198</v>
+        <v>207</v>
       </c>
       <c r="F10" t="s">
-        <v>199</v>
+        <v>208</v>
       </c>
       <c r="G10" t="s">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="H10" t="s">
-        <v>201</v>
+        <v>210</v>
       </c>
       <c r="I10"/>
       <c r="J10" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="K10" t="s">
-        <v>203</v>
+        <v>212</v>
       </c>
       <c r="L10" t="s">
-        <v>204</v>
+        <v>213</v>
       </c>
       <c r="M10" t="s">
-        <v>205</v>
+        <v>214</v>
       </c>
       <c r="N10" t="n">
         <v>1</v>
       </c>
       <c r="O10" t="s">
-        <v>206</v>
+        <v>215</v>
       </c>
       <c r="P10" t="n">
         <v>1.667</v>
@@ -2811,79 +3439,82 @@
         <v>20</v>
       </c>
       <c r="T10" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="U10" t="s">
-        <v>208</v>
+        <v>217</v>
       </c>
       <c r="V10"/>
       <c r="W10"/>
       <c r="X10" t="s">
-        <v>209</v>
+        <v>218</v>
       </c>
       <c r="Y10" t="s">
-        <v>210</v>
+        <v>219</v>
       </c>
       <c r="Z10" t="s">
-        <v>211</v>
+        <v>220</v>
       </c>
       <c r="AA10"/>
       <c r="AB10" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="AC10" t="n">
         <v>30</v>
       </c>
       <c r="AD10"/>
       <c r="AE10" t="s">
-        <v>213</v>
+        <v>222</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B11" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="C11" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="D11" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="E11" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="F11" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="G11" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="H11" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="I11" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="J11" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="K11" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="L11" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="M11" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="N11" t="n">
         <v>1</v>
       </c>
       <c r="O11" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="P11" t="n">
         <v>1.909</v>
@@ -2896,32 +3527,187 @@
         <v>18.18</v>
       </c>
       <c r="T11" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="U11" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="V11"/>
       <c r="W11"/>
       <c r="X11" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="Y11" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="Z11" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
       <c r="AA11"/>
       <c r="AB11" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
       <c r="AC11" t="n">
         <v>20</v>
       </c>
       <c r="AD11"/>
       <c r="AE11" t="s">
-        <v>234</v>
+        <v>244</v>
+      </c>
+      <c r="AF11" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>246</v>
+      </c>
+      <c r="B12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D12" t="s">
+        <v>249</v>
+      </c>
+      <c r="E12" t="s">
+        <v>250</v>
+      </c>
+      <c r="F12" t="s">
+        <v>251</v>
+      </c>
+      <c r="G12" t="s">
+        <v>252</v>
+      </c>
+      <c r="H12" t="s">
+        <v>253</v>
+      </c>
+      <c r="I12"/>
+      <c r="J12" t="s">
+        <v>254</v>
+      </c>
+      <c r="K12" t="s">
+        <v>255</v>
+      </c>
+      <c r="L12" t="s">
+        <v>256</v>
+      </c>
+      <c r="M12" t="s">
+        <v>257</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12"/>
+      <c r="P12"/>
+      <c r="Q12"/>
+      <c r="R12"/>
+      <c r="S12"/>
+      <c r="T12" t="s">
+        <v>258</v>
+      </c>
+      <c r="U12" t="s">
+        <v>259</v>
+      </c>
+      <c r="V12"/>
+      <c r="W12"/>
+      <c r="X12" t="s">
+        <v>260</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>261</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>262</v>
+      </c>
+      <c r="AA12"/>
+      <c r="AB12" t="s">
+        <v>263</v>
+      </c>
+      <c r="AC12"/>
+      <c r="AD12"/>
+      <c r="AE12" t="s">
+        <v>264</v>
+      </c>
+      <c r="AF12" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>266</v>
+      </c>
+      <c r="B13" t="s">
+        <v>267</v>
+      </c>
+      <c r="C13" t="s">
+        <v>268</v>
+      </c>
+      <c r="D13" t="s">
+        <v>269</v>
+      </c>
+      <c r="E13" t="s">
+        <v>270</v>
+      </c>
+      <c r="F13" t="s">
+        <v>271</v>
+      </c>
+      <c r="G13" t="s">
+        <v>272</v>
+      </c>
+      <c r="H13" t="s">
+        <v>273</v>
+      </c>
+      <c r="I13"/>
+      <c r="J13" t="s">
+        <v>274</v>
+      </c>
+      <c r="K13" t="s">
+        <v>275</v>
+      </c>
+      <c r="L13" t="s">
+        <v>276</v>
+      </c>
+      <c r="M13" t="s">
+        <v>277</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13"/>
+      <c r="P13"/>
+      <c r="Q13"/>
+      <c r="R13"/>
+      <c r="S13"/>
+      <c r="T13" t="s">
+        <v>278</v>
+      </c>
+      <c r="U13" t="s">
+        <v>279</v>
+      </c>
+      <c r="V13"/>
+      <c r="W13"/>
+      <c r="X13" t="s">
+        <v>280</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>281</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>282</v>
+      </c>
+      <c r="AA13"/>
+      <c r="AB13" t="s">
+        <v>283</v>
+      </c>
+      <c r="AC13"/>
+      <c r="AD13"/>
+      <c r="AE13" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF13" t="s">
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -2933,178 +3719,178 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>235</v>
+        <v>286</v>
       </c>
       <c r="B1" t="s">
-        <v>236</v>
+        <v>287</v>
       </c>
       <c r="C1" t="s">
-        <v>237</v>
+        <v>288</v>
       </c>
       <c r="D1" t="s">
-        <v>238</v>
+        <v>289</v>
       </c>
       <c r="E1" t="s">
-        <v>239</v>
+        <v>290</v>
       </c>
       <c r="F1" t="s">
-        <v>240</v>
+        <v>291</v>
       </c>
       <c r="G1" t="s">
-        <v>241</v>
+        <v>292</v>
       </c>
       <c r="H1" t="s">
-        <v>242</v>
+        <v>293</v>
       </c>
       <c r="I1" t="s">
-        <v>243</v>
+        <v>294</v>
       </c>
       <c r="J1" t="s">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="K1" t="s">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="L1" t="s">
-        <v>246</v>
+        <v>297</v>
       </c>
       <c r="M1" t="s">
-        <v>247</v>
+        <v>298</v>
       </c>
       <c r="N1" t="s">
-        <v>248</v>
+        <v>299</v>
       </c>
       <c r="O1" t="s">
-        <v>249</v>
+        <v>300</v>
       </c>
       <c r="P1" t="s">
-        <v>250</v>
+        <v>301</v>
       </c>
       <c r="Q1" t="s">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="R1" t="s">
-        <v>252</v>
+        <v>303</v>
       </c>
       <c r="S1" t="s">
-        <v>253</v>
+        <v>304</v>
       </c>
       <c r="T1" t="s">
-        <v>254</v>
+        <v>305</v>
       </c>
       <c r="U1" t="s">
-        <v>255</v>
+        <v>306</v>
       </c>
       <c r="V1" t="s">
-        <v>256</v>
+        <v>307</v>
       </c>
       <c r="W1" t="s">
-        <v>257</v>
+        <v>308</v>
       </c>
       <c r="X1" t="s">
-        <v>258</v>
+        <v>309</v>
       </c>
       <c r="Y1" t="s">
-        <v>259</v>
+        <v>310</v>
       </c>
       <c r="Z1" t="s">
-        <v>260</v>
+        <v>311</v>
       </c>
       <c r="AA1" t="s">
-        <v>261</v>
+        <v>312</v>
       </c>
       <c r="AB1" t="s">
-        <v>262</v>
+        <v>313</v>
       </c>
       <c r="AC1" t="s">
-        <v>263</v>
+        <v>314</v>
       </c>
       <c r="AD1" t="s">
-        <v>264</v>
+        <v>315</v>
       </c>
       <c r="AE1" t="s">
-        <v>265</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>266</v>
+        <v>317</v>
       </c>
       <c r="B2" t="s">
-        <v>267</v>
+        <v>318</v>
       </c>
       <c r="C2" t="s">
-        <v>268</v>
+        <v>319</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>269</v>
+        <v>320</v>
       </c>
       <c r="F2" t="s">
-        <v>270</v>
+        <v>321</v>
       </c>
       <c r="G2" t="s">
-        <v>271</v>
+        <v>322</v>
       </c>
       <c r="H2" t="s">
-        <v>272</v>
+        <v>323</v>
       </c>
       <c r="I2" t="s">
-        <v>273</v>
+        <v>324</v>
       </c>
       <c r="J2" t="s">
-        <v>274</v>
+        <v>325</v>
       </c>
       <c r="K2" t="s">
-        <v>275</v>
+        <v>326</v>
       </c>
       <c r="L2" t="s">
-        <v>276</v>
+        <v>327</v>
       </c>
       <c r="M2" t="s">
-        <v>277</v>
+        <v>328</v>
       </c>
       <c r="N2" t="s">
-        <v>278</v>
+        <v>329</v>
       </c>
       <c r="O2" t="s">
-        <v>279</v>
+        <v>330</v>
       </c>
       <c r="P2" t="s">
-        <v>280</v>
+        <v>331</v>
       </c>
       <c r="Q2" t="s">
-        <v>281</v>
+        <v>332</v>
       </c>
       <c r="R2"/>
       <c r="S2" t="s">
-        <v>282</v>
+        <v>333</v>
       </c>
       <c r="T2" t="s">
-        <v>283</v>
+        <v>334</v>
       </c>
       <c r="U2" t="s">
-        <v>284</v>
+        <v>335</v>
       </c>
       <c r="V2" t="s">
-        <v>285</v>
+        <v>336</v>
       </c>
       <c r="W2" t="s">
-        <v>286</v>
+        <v>337</v>
       </c>
       <c r="X2" t="s">
-        <v>287</v>
+        <v>338</v>
       </c>
       <c r="Y2" t="s">
-        <v>288</v>
+        <v>339</v>
       </c>
       <c r="Z2" t="s">
-        <v>289</v>
+        <v>340</v>
       </c>
       <c r="AA2" t="s">
-        <v>290</v>
+        <v>341</v>
       </c>
       <c r="AB2" t="n">
         <v>2</v>
@@ -3113,93 +3899,93 @@
         <v>1</v>
       </c>
       <c r="AD2" t="s">
-        <v>291</v>
+        <v>342</v>
       </c>
       <c r="AE2" t="s">
-        <v>292</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>293</v>
+        <v>344</v>
       </c>
       <c r="B3" t="s">
-        <v>294</v>
+        <v>345</v>
       </c>
       <c r="C3" t="s">
-        <v>295</v>
+        <v>346</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>296</v>
+        <v>347</v>
       </c>
       <c r="F3" t="s">
-        <v>297</v>
+        <v>348</v>
       </c>
       <c r="G3" t="s">
-        <v>298</v>
+        <v>349</v>
       </c>
       <c r="H3" t="s">
-        <v>299</v>
+        <v>350</v>
       </c>
       <c r="I3" t="s">
-        <v>300</v>
+        <v>351</v>
       </c>
       <c r="J3" t="s">
-        <v>301</v>
+        <v>352</v>
       </c>
       <c r="K3" t="s">
-        <v>302</v>
+        <v>353</v>
       </c>
       <c r="L3" t="s">
-        <v>303</v>
+        <v>354</v>
       </c>
       <c r="M3" t="s">
-        <v>304</v>
+        <v>355</v>
       </c>
       <c r="N3" t="s">
-        <v>305</v>
+        <v>356</v>
       </c>
       <c r="O3" t="s">
-        <v>306</v>
+        <v>357</v>
       </c>
       <c r="P3" t="s">
-        <v>307</v>
+        <v>358</v>
       </c>
       <c r="Q3" t="s">
-        <v>308</v>
+        <v>359</v>
       </c>
       <c r="R3" t="s">
-        <v>309</v>
+        <v>360</v>
       </c>
       <c r="S3" t="s">
-        <v>310</v>
+        <v>361</v>
       </c>
       <c r="T3" t="s">
-        <v>311</v>
+        <v>362</v>
       </c>
       <c r="U3" t="s">
-        <v>312</v>
+        <v>363</v>
       </c>
       <c r="V3" t="s">
-        <v>313</v>
+        <v>364</v>
       </c>
       <c r="W3" t="s">
-        <v>314</v>
+        <v>365</v>
       </c>
       <c r="X3" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
       <c r="Y3" t="s">
-        <v>316</v>
+        <v>367</v>
       </c>
       <c r="Z3" t="s">
-        <v>317</v>
+        <v>368</v>
       </c>
       <c r="AA3" t="s">
-        <v>318</v>
+        <v>369</v>
       </c>
       <c r="AB3" t="n">
         <v>2</v>
@@ -3208,91 +3994,91 @@
         <v>1</v>
       </c>
       <c r="AD3" t="s">
-        <v>319</v>
+        <v>370</v>
       </c>
       <c r="AE3" t="s">
-        <v>320</v>
+        <v>371</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>321</v>
+        <v>372</v>
       </c>
       <c r="B4" t="s">
-        <v>322</v>
+        <v>373</v>
       </c>
       <c r="C4" t="s">
-        <v>323</v>
+        <v>374</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>324</v>
+        <v>375</v>
       </c>
       <c r="F4" t="s">
-        <v>325</v>
+        <v>376</v>
       </c>
       <c r="G4" t="s">
-        <v>326</v>
+        <v>377</v>
       </c>
       <c r="H4" t="s">
-        <v>327</v>
+        <v>378</v>
       </c>
       <c r="I4" t="s">
-        <v>328</v>
+        <v>379</v>
       </c>
       <c r="J4" t="s">
-        <v>329</v>
+        <v>380</v>
       </c>
       <c r="K4" t="s">
-        <v>330</v>
+        <v>381</v>
       </c>
       <c r="L4" t="s">
-        <v>331</v>
+        <v>382</v>
       </c>
       <c r="M4" t="s">
-        <v>332</v>
+        <v>383</v>
       </c>
       <c r="N4" t="s">
-        <v>333</v>
+        <v>384</v>
       </c>
       <c r="O4" t="s">
-        <v>334</v>
+        <v>385</v>
       </c>
       <c r="P4" t="s">
-        <v>335</v>
+        <v>386</v>
       </c>
       <c r="Q4" t="s">
-        <v>336</v>
+        <v>387</v>
       </c>
       <c r="R4"/>
       <c r="S4" t="s">
-        <v>337</v>
+        <v>388</v>
       </c>
       <c r="T4" t="s">
-        <v>338</v>
+        <v>389</v>
       </c>
       <c r="U4" t="s">
-        <v>339</v>
+        <v>390</v>
       </c>
       <c r="V4" t="s">
-        <v>340</v>
+        <v>391</v>
       </c>
       <c r="W4" t="s">
-        <v>341</v>
+        <v>392</v>
       </c>
       <c r="X4" t="s">
-        <v>342</v>
+        <v>393</v>
       </c>
       <c r="Y4" t="s">
-        <v>343</v>
+        <v>394</v>
       </c>
       <c r="Z4" t="s">
-        <v>344</v>
+        <v>395</v>
       </c>
       <c r="AA4" t="s">
-        <v>345</v>
+        <v>396</v>
       </c>
       <c r="AB4" t="n">
         <v>2</v>
@@ -3301,91 +4087,91 @@
         <v>1</v>
       </c>
       <c r="AD4" t="s">
-        <v>346</v>
+        <v>397</v>
       </c>
       <c r="AE4" t="s">
-        <v>347</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>348</v>
+        <v>399</v>
       </c>
       <c r="B5" t="s">
-        <v>349</v>
+        <v>400</v>
       </c>
       <c r="C5" t="s">
-        <v>350</v>
+        <v>401</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>351</v>
+        <v>402</v>
       </c>
       <c r="F5" t="s">
-        <v>352</v>
+        <v>403</v>
       </c>
       <c r="G5" t="s">
-        <v>353</v>
+        <v>404</v>
       </c>
       <c r="H5" t="s">
-        <v>354</v>
+        <v>405</v>
       </c>
       <c r="I5" t="s">
-        <v>355</v>
+        <v>406</v>
       </c>
       <c r="J5"/>
       <c r="K5" t="s">
-        <v>356</v>
+        <v>407</v>
       </c>
       <c r="L5" t="s">
-        <v>357</v>
+        <v>408</v>
       </c>
       <c r="M5" t="s">
-        <v>358</v>
+        <v>409</v>
       </c>
       <c r="N5" t="s">
-        <v>359</v>
+        <v>410</v>
       </c>
       <c r="O5" t="s">
-        <v>360</v>
+        <v>411</v>
       </c>
       <c r="P5" t="s">
-        <v>361</v>
+        <v>412</v>
       </c>
       <c r="Q5" t="s">
-        <v>362</v>
+        <v>413</v>
       </c>
       <c r="R5" t="s">
-        <v>363</v>
+        <v>414</v>
       </c>
       <c r="S5" t="s">
-        <v>364</v>
+        <v>415</v>
       </c>
       <c r="T5" t="s">
-        <v>365</v>
+        <v>416</v>
       </c>
       <c r="U5" t="s">
-        <v>366</v>
+        <v>417</v>
       </c>
       <c r="V5" t="s">
-        <v>367</v>
+        <v>418</v>
       </c>
       <c r="W5" t="s">
-        <v>368</v>
+        <v>419</v>
       </c>
       <c r="X5" t="s">
-        <v>369</v>
+        <v>420</v>
       </c>
       <c r="Y5" t="s">
-        <v>370</v>
+        <v>421</v>
       </c>
       <c r="Z5" t="s">
-        <v>371</v>
+        <v>422</v>
       </c>
       <c r="AA5" t="s">
-        <v>372</v>
+        <v>423</v>
       </c>
       <c r="AB5" t="n">
         <v>2</v>
@@ -3394,93 +4180,93 @@
         <v>1</v>
       </c>
       <c r="AD5" t="s">
-        <v>373</v>
+        <v>424</v>
       </c>
       <c r="AE5" t="s">
-        <v>374</v>
+        <v>425</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>375</v>
+        <v>426</v>
       </c>
       <c r="B6" t="s">
-        <v>376</v>
+        <v>427</v>
       </c>
       <c r="C6" t="s">
-        <v>377</v>
+        <v>428</v>
       </c>
       <c r="D6" t="n">
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>378</v>
+        <v>429</v>
       </c>
       <c r="F6" t="s">
-        <v>379</v>
+        <v>430</v>
       </c>
       <c r="G6" t="s">
-        <v>380</v>
+        <v>431</v>
       </c>
       <c r="H6" t="s">
-        <v>381</v>
+        <v>432</v>
       </c>
       <c r="I6" t="s">
-        <v>382</v>
+        <v>433</v>
       </c>
       <c r="J6" t="s">
-        <v>383</v>
+        <v>434</v>
       </c>
       <c r="K6" t="s">
-        <v>384</v>
+        <v>435</v>
       </c>
       <c r="L6" t="s">
-        <v>385</v>
+        <v>436</v>
       </c>
       <c r="M6" t="s">
-        <v>386</v>
+        <v>437</v>
       </c>
       <c r="N6" t="s">
-        <v>387</v>
+        <v>438</v>
       </c>
       <c r="O6" t="s">
-        <v>388</v>
+        <v>439</v>
       </c>
       <c r="P6" t="s">
-        <v>389</v>
+        <v>440</v>
       </c>
       <c r="Q6" t="s">
-        <v>390</v>
+        <v>441</v>
       </c>
       <c r="R6" t="s">
-        <v>391</v>
+        <v>442</v>
       </c>
       <c r="S6" t="s">
-        <v>392</v>
+        <v>443</v>
       </c>
       <c r="T6" t="s">
-        <v>393</v>
+        <v>444</v>
       </c>
       <c r="U6" t="s">
-        <v>394</v>
+        <v>445</v>
       </c>
       <c r="V6" t="s">
-        <v>395</v>
+        <v>446</v>
       </c>
       <c r="W6" t="s">
-        <v>396</v>
+        <v>447</v>
       </c>
       <c r="X6" t="s">
-        <v>397</v>
+        <v>448</v>
       </c>
       <c r="Y6" t="s">
-        <v>398</v>
+        <v>449</v>
       </c>
       <c r="Z6" t="s">
-        <v>399</v>
+        <v>450</v>
       </c>
       <c r="AA6" t="s">
-        <v>400</v>
+        <v>451</v>
       </c>
       <c r="AB6" t="n">
         <v>2</v>
@@ -3489,93 +4275,93 @@
         <v>1</v>
       </c>
       <c r="AD6" t="s">
-        <v>401</v>
+        <v>452</v>
       </c>
       <c r="AE6" t="s">
-        <v>402</v>
+        <v>453</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>403</v>
+        <v>454</v>
       </c>
       <c r="B7" t="s">
-        <v>404</v>
+        <v>455</v>
       </c>
       <c r="C7" t="s">
-        <v>405</v>
+        <v>456</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>406</v>
+        <v>457</v>
       </c>
       <c r="F7" t="s">
-        <v>407</v>
+        <v>458</v>
       </c>
       <c r="G7" t="s">
-        <v>408</v>
+        <v>459</v>
       </c>
       <c r="H7" t="s">
-        <v>409</v>
+        <v>460</v>
       </c>
       <c r="I7" t="s">
-        <v>410</v>
+        <v>461</v>
       </c>
       <c r="J7" t="s">
-        <v>411</v>
+        <v>462</v>
       </c>
       <c r="K7" t="s">
-        <v>412</v>
+        <v>463</v>
       </c>
       <c r="L7" t="s">
-        <v>413</v>
+        <v>464</v>
       </c>
       <c r="M7" t="s">
-        <v>414</v>
+        <v>465</v>
       </c>
       <c r="N7" t="s">
-        <v>415</v>
+        <v>466</v>
       </c>
       <c r="O7" t="s">
-        <v>416</v>
+        <v>467</v>
       </c>
       <c r="P7" t="s">
-        <v>417</v>
+        <v>468</v>
       </c>
       <c r="Q7" t="s">
-        <v>418</v>
+        <v>469</v>
       </c>
       <c r="R7" t="s">
-        <v>419</v>
+        <v>470</v>
       </c>
       <c r="S7" t="s">
-        <v>420</v>
+        <v>471</v>
       </c>
       <c r="T7" t="s">
-        <v>421</v>
+        <v>472</v>
       </c>
       <c r="U7" t="s">
-        <v>422</v>
+        <v>473</v>
       </c>
       <c r="V7" t="s">
-        <v>423</v>
+        <v>474</v>
       </c>
       <c r="W7" t="s">
-        <v>424</v>
+        <v>475</v>
       </c>
       <c r="X7" t="s">
-        <v>425</v>
+        <v>476</v>
       </c>
       <c r="Y7" t="s">
-        <v>426</v>
+        <v>477</v>
       </c>
       <c r="Z7" t="s">
-        <v>427</v>
+        <v>478</v>
       </c>
       <c r="AA7" t="s">
-        <v>428</v>
+        <v>479</v>
       </c>
       <c r="AB7" t="n">
         <v>2</v>
@@ -3584,89 +4370,89 @@
         <v>1</v>
       </c>
       <c r="AD7" t="s">
-        <v>429</v>
+        <v>480</v>
       </c>
       <c r="AE7" t="s">
-        <v>430</v>
+        <v>481</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>431</v>
+        <v>482</v>
       </c>
       <c r="B8" t="s">
-        <v>432</v>
+        <v>483</v>
       </c>
       <c r="C8" t="s">
-        <v>433</v>
+        <v>484</v>
       </c>
       <c r="D8" t="n">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>434</v>
+        <v>485</v>
       </c>
       <c r="F8" t="s">
-        <v>435</v>
+        <v>486</v>
       </c>
       <c r="G8" t="s">
-        <v>436</v>
+        <v>487</v>
       </c>
       <c r="H8" t="s">
-        <v>437</v>
+        <v>488</v>
       </c>
       <c r="I8" t="s">
-        <v>438</v>
+        <v>489</v>
       </c>
       <c r="J8"/>
       <c r="K8" t="s">
-        <v>439</v>
+        <v>490</v>
       </c>
       <c r="L8" t="s">
-        <v>440</v>
+        <v>491</v>
       </c>
       <c r="M8" t="s">
-        <v>441</v>
+        <v>492</v>
       </c>
       <c r="N8" t="s">
-        <v>442</v>
+        <v>493</v>
       </c>
       <c r="O8" t="s">
-        <v>443</v>
+        <v>494</v>
       </c>
       <c r="P8" t="s">
-        <v>444</v>
+        <v>495</v>
       </c>
       <c r="Q8" t="s">
-        <v>445</v>
+        <v>496</v>
       </c>
       <c r="R8"/>
       <c r="S8" t="s">
-        <v>446</v>
+        <v>497</v>
       </c>
       <c r="T8" t="s">
-        <v>447</v>
+        <v>498</v>
       </c>
       <c r="U8" t="s">
-        <v>448</v>
+        <v>499</v>
       </c>
       <c r="V8" t="s">
-        <v>449</v>
+        <v>500</v>
       </c>
       <c r="W8" t="s">
-        <v>450</v>
+        <v>501</v>
       </c>
       <c r="X8" t="s">
-        <v>451</v>
+        <v>502</v>
       </c>
       <c r="Y8" t="s">
-        <v>452</v>
+        <v>503</v>
       </c>
       <c r="Z8" t="s">
-        <v>453</v>
+        <v>504</v>
       </c>
       <c r="AA8" t="s">
-        <v>454</v>
+        <v>505</v>
       </c>
       <c r="AB8" t="n">
         <v>2</v>
@@ -3675,93 +4461,93 @@
         <v>1</v>
       </c>
       <c r="AD8" t="s">
-        <v>455</v>
+        <v>506</v>
       </c>
       <c r="AE8" t="s">
-        <v>456</v>
+        <v>507</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>457</v>
+        <v>508</v>
       </c>
       <c r="B9" t="s">
-        <v>458</v>
+        <v>509</v>
       </c>
       <c r="C9" t="s">
-        <v>459</v>
+        <v>510</v>
       </c>
       <c r="D9" t="n">
         <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>460</v>
+        <v>511</v>
       </c>
       <c r="F9" t="s">
-        <v>461</v>
+        <v>512</v>
       </c>
       <c r="G9" t="s">
-        <v>462</v>
+        <v>513</v>
       </c>
       <c r="H9" t="s">
-        <v>463</v>
+        <v>514</v>
       </c>
       <c r="I9" t="s">
-        <v>464</v>
+        <v>515</v>
       </c>
       <c r="J9" t="s">
-        <v>465</v>
+        <v>516</v>
       </c>
       <c r="K9" t="s">
-        <v>466</v>
+        <v>517</v>
       </c>
       <c r="L9" t="s">
-        <v>467</v>
+        <v>518</v>
       </c>
       <c r="M9" t="s">
-        <v>468</v>
+        <v>519</v>
       </c>
       <c r="N9" t="s">
-        <v>469</v>
+        <v>520</v>
       </c>
       <c r="O9" t="s">
-        <v>470</v>
+        <v>521</v>
       </c>
       <c r="P9" t="s">
-        <v>471</v>
+        <v>522</v>
       </c>
       <c r="Q9" t="s">
-        <v>472</v>
+        <v>523</v>
       </c>
       <c r="R9" t="s">
-        <v>473</v>
+        <v>524</v>
       </c>
       <c r="S9" t="s">
-        <v>474</v>
+        <v>525</v>
       </c>
       <c r="T9" t="s">
-        <v>475</v>
+        <v>526</v>
       </c>
       <c r="U9" t="s">
-        <v>476</v>
+        <v>527</v>
       </c>
       <c r="V9" t="s">
-        <v>477</v>
+        <v>528</v>
       </c>
       <c r="W9" t="s">
-        <v>478</v>
+        <v>529</v>
       </c>
       <c r="X9" t="s">
-        <v>479</v>
+        <v>530</v>
       </c>
       <c r="Y9" t="s">
-        <v>480</v>
+        <v>531</v>
       </c>
       <c r="Z9" t="s">
-        <v>481</v>
+        <v>532</v>
       </c>
       <c r="AA9" t="s">
-        <v>482</v>
+        <v>533</v>
       </c>
       <c r="AB9" t="n">
         <v>2</v>
@@ -3770,10 +4556,10 @@
         <v>1</v>
       </c>
       <c r="AD9" t="s">
-        <v>483</v>
+        <v>534</v>
       </c>
       <c r="AE9" t="s">
-        <v>484</v>
+        <v>535</v>
       </c>
     </row>
   </sheetData>
@@ -3785,547 +4571,547 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>485</v>
+        <v>536</v>
       </c>
       <c r="B1" t="s">
-        <v>486</v>
+        <v>537</v>
       </c>
       <c r="C1" t="s">
-        <v>487</v>
+        <v>538</v>
       </c>
       <c r="D1" t="s">
-        <v>488</v>
+        <v>539</v>
       </c>
       <c r="E1" t="s">
-        <v>489</v>
+        <v>540</v>
       </c>
       <c r="F1" t="s">
-        <v>490</v>
+        <v>541</v>
       </c>
       <c r="G1" t="s">
-        <v>491</v>
+        <v>542</v>
       </c>
       <c r="H1" t="s">
-        <v>492</v>
+        <v>543</v>
       </c>
       <c r="I1" t="s">
-        <v>493</v>
+        <v>544</v>
       </c>
       <c r="J1" t="s">
-        <v>494</v>
+        <v>545</v>
       </c>
       <c r="K1" t="s">
-        <v>495</v>
+        <v>546</v>
       </c>
       <c r="L1" t="s">
-        <v>496</v>
+        <v>547</v>
       </c>
       <c r="M1" t="s">
-        <v>497</v>
+        <v>548</v>
       </c>
       <c r="N1" t="s">
-        <v>498</v>
+        <v>549</v>
       </c>
       <c r="O1" t="s">
-        <v>499</v>
+        <v>550</v>
       </c>
       <c r="P1" t="s">
-        <v>500</v>
+        <v>551</v>
       </c>
       <c r="Q1" t="s">
-        <v>501</v>
+        <v>552</v>
       </c>
       <c r="R1" t="s">
-        <v>502</v>
+        <v>553</v>
       </c>
       <c r="S1" t="s">
-        <v>503</v>
+        <v>554</v>
       </c>
       <c r="T1" t="s">
-        <v>504</v>
+        <v>555</v>
       </c>
       <c r="U1" t="s">
-        <v>505</v>
+        <v>556</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>506</v>
+        <v>557</v>
       </c>
       <c r="B2" t="s">
-        <v>507</v>
+        <v>558</v>
       </c>
       <c r="C2" t="s">
-        <v>508</v>
+        <v>559</v>
       </c>
       <c r="D2" t="s">
-        <v>509</v>
+        <v>560</v>
       </c>
       <c r="E2" t="s">
-        <v>510</v>
+        <v>561</v>
       </c>
       <c r="F2" t="s">
-        <v>511</v>
+        <v>562</v>
       </c>
       <c r="G2" t="s">
-        <v>512</v>
+        <v>563</v>
       </c>
       <c r="H2" t="s">
-        <v>513</v>
+        <v>564</v>
       </c>
       <c r="I2" t="s">
-        <v>514</v>
+        <v>565</v>
       </c>
       <c r="J2" t="s">
-        <v>515</v>
+        <v>566</v>
       </c>
       <c r="K2"/>
       <c r="L2" t="n">
         <v>82</v>
       </c>
       <c r="M2" t="s">
-        <v>516</v>
+        <v>567</v>
       </c>
       <c r="N2" t="s">
-        <v>517</v>
+        <v>568</v>
       </c>
       <c r="O2" t="s">
-        <v>518</v>
+        <v>569</v>
       </c>
       <c r="P2" t="s">
-        <v>519</v>
+        <v>570</v>
       </c>
       <c r="Q2" t="s">
-        <v>520</v>
+        <v>571</v>
       </c>
       <c r="R2" t="s">
-        <v>521</v>
+        <v>572</v>
       </c>
       <c r="S2" t="s">
-        <v>522</v>
+        <v>573</v>
       </c>
       <c r="T2" t="s">
-        <v>523</v>
+        <v>574</v>
       </c>
       <c r="U2"/>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>524</v>
+        <v>575</v>
       </c>
       <c r="B3" t="s">
-        <v>525</v>
+        <v>576</v>
       </c>
       <c r="C3" t="s">
-        <v>526</v>
+        <v>577</v>
       </c>
       <c r="D3" t="s">
-        <v>527</v>
+        <v>578</v>
       </c>
       <c r="E3" t="s">
-        <v>528</v>
+        <v>579</v>
       </c>
       <c r="F3" t="s">
-        <v>529</v>
+        <v>580</v>
       </c>
       <c r="G3" t="s">
-        <v>530</v>
+        <v>581</v>
       </c>
       <c r="H3" t="s">
-        <v>531</v>
+        <v>582</v>
       </c>
       <c r="I3" t="s">
-        <v>532</v>
+        <v>583</v>
       </c>
       <c r="J3" t="s">
-        <v>533</v>
+        <v>584</v>
       </c>
       <c r="K3"/>
       <c r="L3" t="n">
         <v>91</v>
       </c>
       <c r="M3" t="s">
-        <v>534</v>
+        <v>585</v>
       </c>
       <c r="N3" t="s">
-        <v>535</v>
+        <v>586</v>
       </c>
       <c r="O3"/>
       <c r="P3" t="s">
-        <v>536</v>
+        <v>587</v>
       </c>
       <c r="Q3" t="s">
-        <v>537</v>
+        <v>588</v>
       </c>
       <c r="R3" t="s">
-        <v>538</v>
+        <v>589</v>
       </c>
       <c r="S3" t="s">
-        <v>539</v>
+        <v>590</v>
       </c>
       <c r="T3" t="s">
-        <v>540</v>
+        <v>591</v>
       </c>
       <c r="U3"/>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>541</v>
+        <v>592</v>
       </c>
       <c r="B4" t="s">
-        <v>542</v>
+        <v>593</v>
       </c>
       <c r="C4" t="s">
-        <v>543</v>
+        <v>594</v>
       </c>
       <c r="D4" t="s">
-        <v>544</v>
+        <v>595</v>
       </c>
       <c r="E4" t="s">
-        <v>545</v>
+        <v>596</v>
       </c>
       <c r="F4" t="s">
-        <v>546</v>
+        <v>597</v>
       </c>
       <c r="G4" t="s">
-        <v>547</v>
+        <v>598</v>
       </c>
       <c r="H4" t="s">
-        <v>548</v>
+        <v>599</v>
       </c>
       <c r="I4" t="s">
-        <v>549</v>
+        <v>600</v>
       </c>
       <c r="J4" t="s">
-        <v>550</v>
+        <v>601</v>
       </c>
       <c r="K4"/>
       <c r="L4" t="n">
         <v>74</v>
       </c>
       <c r="M4" t="s">
-        <v>551</v>
+        <v>602</v>
       </c>
       <c r="N4" t="s">
-        <v>552</v>
+        <v>603</v>
       </c>
       <c r="O4" t="s">
-        <v>553</v>
+        <v>604</v>
       </c>
       <c r="P4" t="s">
-        <v>554</v>
+        <v>605</v>
       </c>
       <c r="Q4" t="s">
-        <v>555</v>
+        <v>606</v>
       </c>
       <c r="R4" t="s">
-        <v>556</v>
+        <v>607</v>
       </c>
       <c r="S4" t="s">
-        <v>557</v>
+        <v>608</v>
       </c>
       <c r="T4" t="s">
-        <v>558</v>
+        <v>609</v>
       </c>
       <c r="U4"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>559</v>
+        <v>610</v>
       </c>
       <c r="B5" t="s">
-        <v>560</v>
+        <v>611</v>
       </c>
       <c r="C5" t="s">
-        <v>561</v>
+        <v>612</v>
       </c>
       <c r="D5" t="s">
-        <v>562</v>
+        <v>613</v>
       </c>
       <c r="E5" t="s">
-        <v>563</v>
+        <v>614</v>
       </c>
       <c r="F5" t="s">
-        <v>564</v>
+        <v>615</v>
       </c>
       <c r="G5" t="s">
-        <v>565</v>
+        <v>616</v>
       </c>
       <c r="H5" t="s">
-        <v>566</v>
+        <v>617</v>
       </c>
       <c r="I5" t="s">
-        <v>567</v>
+        <v>618</v>
       </c>
       <c r="J5" t="s">
-        <v>568</v>
+        <v>619</v>
       </c>
       <c r="K5"/>
       <c r="L5" t="n">
         <v>88</v>
       </c>
       <c r="M5" t="s">
-        <v>569</v>
+        <v>620</v>
       </c>
       <c r="N5" t="s">
-        <v>570</v>
+        <v>621</v>
       </c>
       <c r="O5" t="s">
-        <v>571</v>
+        <v>622</v>
       </c>
       <c r="P5" t="s">
-        <v>572</v>
+        <v>623</v>
       </c>
       <c r="Q5" t="s">
-        <v>573</v>
+        <v>624</v>
       </c>
       <c r="R5" t="s">
-        <v>574</v>
+        <v>625</v>
       </c>
       <c r="S5" t="s">
-        <v>575</v>
+        <v>626</v>
       </c>
       <c r="T5" t="s">
-        <v>576</v>
+        <v>627</v>
       </c>
       <c r="U5"/>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>577</v>
+        <v>628</v>
       </c>
       <c r="B6" t="s">
-        <v>578</v>
+        <v>629</v>
       </c>
       <c r="C6" t="s">
-        <v>579</v>
+        <v>630</v>
       </c>
       <c r="D6" t="s">
-        <v>580</v>
+        <v>631</v>
       </c>
       <c r="E6" t="s">
-        <v>581</v>
+        <v>632</v>
       </c>
       <c r="F6" t="s">
-        <v>582</v>
+        <v>633</v>
       </c>
       <c r="G6" t="s">
-        <v>583</v>
+        <v>634</v>
       </c>
       <c r="H6" t="s">
-        <v>584</v>
+        <v>635</v>
       </c>
       <c r="I6" t="s">
-        <v>585</v>
+        <v>636</v>
       </c>
       <c r="J6" t="s">
-        <v>586</v>
+        <v>637</v>
       </c>
       <c r="K6"/>
       <c r="L6" t="n">
         <v>76</v>
       </c>
       <c r="M6" t="s">
-        <v>587</v>
+        <v>638</v>
       </c>
       <c r="N6" t="s">
-        <v>588</v>
+        <v>639</v>
       </c>
       <c r="O6"/>
       <c r="P6" t="s">
-        <v>589</v>
+        <v>640</v>
       </c>
       <c r="Q6" t="s">
-        <v>590</v>
+        <v>641</v>
       </c>
       <c r="R6" t="s">
-        <v>591</v>
+        <v>642</v>
       </c>
       <c r="S6" t="s">
-        <v>592</v>
+        <v>643</v>
       </c>
       <c r="T6" t="s">
-        <v>593</v>
+        <v>644</v>
       </c>
       <c r="U6"/>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>594</v>
+        <v>645</v>
       </c>
       <c r="B7" t="s">
-        <v>595</v>
+        <v>646</v>
       </c>
       <c r="C7" t="s">
-        <v>596</v>
+        <v>647</v>
       </c>
       <c r="D7" t="s">
-        <v>597</v>
+        <v>648</v>
       </c>
       <c r="E7" t="s">
-        <v>598</v>
+        <v>649</v>
       </c>
       <c r="F7" t="s">
-        <v>599</v>
+        <v>650</v>
       </c>
       <c r="G7" t="s">
-        <v>600</v>
+        <v>651</v>
       </c>
       <c r="H7" t="s">
-        <v>601</v>
+        <v>652</v>
       </c>
       <c r="I7" t="s">
-        <v>602</v>
+        <v>653</v>
       </c>
       <c r="J7" t="s">
-        <v>603</v>
+        <v>654</v>
       </c>
       <c r="K7"/>
       <c r="L7" t="n">
         <v>93</v>
       </c>
       <c r="M7" t="s">
-        <v>604</v>
+        <v>655</v>
       </c>
       <c r="N7" t="s">
-        <v>605</v>
+        <v>656</v>
       </c>
       <c r="O7"/>
       <c r="P7" t="s">
-        <v>606</v>
+        <v>657</v>
       </c>
       <c r="Q7" t="s">
-        <v>607</v>
+        <v>658</v>
       </c>
       <c r="R7" t="s">
-        <v>608</v>
+        <v>659</v>
       </c>
       <c r="S7" t="s">
-        <v>609</v>
+        <v>660</v>
       </c>
       <c r="T7" t="s">
-        <v>610</v>
+        <v>661</v>
       </c>
       <c r="U7"/>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>611</v>
+        <v>662</v>
       </c>
       <c r="B8" t="s">
-        <v>612</v>
+        <v>663</v>
       </c>
       <c r="C8" t="s">
-        <v>613</v>
+        <v>664</v>
       </c>
       <c r="D8" t="s">
-        <v>614</v>
+        <v>665</v>
       </c>
       <c r="E8" t="s">
-        <v>615</v>
+        <v>666</v>
       </c>
       <c r="F8" t="s">
-        <v>616</v>
+        <v>667</v>
       </c>
       <c r="G8" t="s">
-        <v>617</v>
+        <v>668</v>
       </c>
       <c r="H8" t="s">
-        <v>618</v>
+        <v>669</v>
       </c>
       <c r="I8" t="s">
-        <v>619</v>
+        <v>670</v>
       </c>
       <c r="J8" t="s">
-        <v>620</v>
+        <v>671</v>
       </c>
       <c r="K8"/>
       <c r="L8" t="n">
         <v>71</v>
       </c>
       <c r="M8" t="s">
-        <v>621</v>
+        <v>672</v>
       </c>
       <c r="N8" t="s">
-        <v>622</v>
+        <v>673</v>
       </c>
       <c r="O8"/>
       <c r="P8" t="s">
-        <v>623</v>
+        <v>674</v>
       </c>
       <c r="Q8" t="s">
-        <v>624</v>
+        <v>675</v>
       </c>
       <c r="R8" t="s">
-        <v>625</v>
+        <v>676</v>
       </c>
       <c r="S8" t="s">
-        <v>626</v>
+        <v>677</v>
       </c>
       <c r="T8" t="s">
-        <v>627</v>
+        <v>678</v>
       </c>
       <c r="U8"/>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>628</v>
+        <v>679</v>
       </c>
       <c r="B9" t="s">
-        <v>629</v>
+        <v>680</v>
       </c>
       <c r="C9" t="s">
-        <v>630</v>
+        <v>681</v>
       </c>
       <c r="D9" t="s">
-        <v>631</v>
+        <v>682</v>
       </c>
       <c r="E9" t="s">
-        <v>632</v>
+        <v>683</v>
       </c>
       <c r="F9" t="s">
-        <v>633</v>
+        <v>684</v>
       </c>
       <c r="G9" t="s">
-        <v>634</v>
+        <v>685</v>
       </c>
       <c r="H9" t="s">
-        <v>635</v>
+        <v>686</v>
       </c>
       <c r="I9" t="s">
-        <v>636</v>
+        <v>687</v>
       </c>
       <c r="J9" t="s">
-        <v>637</v>
+        <v>688</v>
       </c>
       <c r="K9"/>
       <c r="L9" t="n">
         <v>85</v>
       </c>
       <c r="M9" t="s">
-        <v>638</v>
+        <v>689</v>
       </c>
       <c r="N9" t="s">
-        <v>639</v>
+        <v>690</v>
       </c>
       <c r="O9"/>
       <c r="P9" t="s">
-        <v>640</v>
+        <v>691</v>
       </c>
       <c r="Q9" t="s">
-        <v>641</v>
+        <v>692</v>
       </c>
       <c r="R9" t="s">
-        <v>642</v>
+        <v>693</v>
       </c>
       <c r="S9" t="s">
-        <v>643</v>
+        <v>694</v>
       </c>
       <c r="T9" t="s">
-        <v>644</v>
+        <v>695</v>
       </c>
       <c r="U9" t="s">
-        <v>645</v>
+        <v>696</v>
       </c>
     </row>
   </sheetData>
@@ -4337,12 +5123,1302 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>646</v>
+        <v>697</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>647</v>
+        <v>698</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3"/>
+    </row>
+    <row r="4">
+      <c r="A4"/>
+    </row>
+    <row r="5">
+      <c r="A5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>701</v>
+      </c>
+      <c r="B6" t="s">
+        <v>702</v>
+      </c>
+      <c r="C6" t="s">
+        <v>703</v>
+      </c>
+      <c r="D6" t="s">
+        <v>704</v>
+      </c>
+      <c r="E6" t="s">
+        <v>705</v>
+      </c>
+      <c r="F6" t="s">
+        <v>706</v>
+      </c>
+      <c r="G6" t="s">
+        <v>707</v>
+      </c>
+      <c r="H6" t="s">
+        <v>708</v>
+      </c>
+      <c r="I6" t="s">
+        <v>709</v>
+      </c>
+      <c r="J6" t="s">
+        <v>710</v>
+      </c>
+      <c r="K6" t="s">
+        <v>711</v>
+      </c>
+      <c r="L6" t="s">
+        <v>712</v>
+      </c>
+      <c r="M6" t="s">
+        <v>713</v>
+      </c>
+      <c r="N6" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>715</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="C7" t="s">
+        <v>716</v>
+      </c>
+      <c r="D7" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>717</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7"/>
+      <c r="K7"/>
+      <c r="L7"/>
+      <c r="M7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-1.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>718</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>719</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>720</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8"/>
+      <c r="K8"/>
+      <c r="L8"/>
+      <c r="M8" t="n">
+        <v>-2.0</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1.82</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>721</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>722</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="s">
+        <v>723</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9"/>
+      <c r="K9"/>
+      <c r="L9"/>
+      <c r="M9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>724</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>725</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>726</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10"/>
+      <c r="K10"/>
+      <c r="L10"/>
+      <c r="M10"/>
+      <c r="N10" t="n">
+        <v>-2.73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>727</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>728</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="s">
+        <v>729</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11"/>
+      <c r="K11"/>
+      <c r="L11"/>
+      <c r="M11"/>
+      <c r="N11" t="n">
+        <v>1.64</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>730</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C12" t="s">
+        <v>731</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>732</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12"/>
+      <c r="K12"/>
+      <c r="L12"/>
+      <c r="M12"/>
+      <c r="N12" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>733</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C13" t="s">
+        <v>734</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="s">
+        <v>735</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13"/>
+      <c r="K13"/>
+      <c r="L13"/>
+      <c r="M13"/>
+      <c r="N13" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>736</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C14" t="s">
+        <v>737</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>738</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14"/>
+      <c r="K14"/>
+      <c r="L14"/>
+      <c r="M14"/>
+      <c r="N14" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>739</v>
+      </c>
+      <c r="B15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>740</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>741</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15"/>
+      <c r="K15"/>
+      <c r="L15"/>
+      <c r="M15"/>
+      <c r="N15" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>742</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C16" t="s">
+        <v>743</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
+        <v>744</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16"/>
+      <c r="K16"/>
+      <c r="L16"/>
+      <c r="M16"/>
+      <c r="N16" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>745</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>746</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>747</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17"/>
+      <c r="K17"/>
+      <c r="L17"/>
+      <c r="M17"/>
+      <c r="N17" t="n">
+        <v>-0.09</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>748</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C18" t="s">
+        <v>749</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="s">
+        <v>750</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18"/>
+      <c r="K18"/>
+      <c r="L18"/>
+      <c r="M18"/>
+      <c r="N18" t="n">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>751</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C19" t="s">
+        <v>752</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>753</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19"/>
+      <c r="K19"/>
+      <c r="L19"/>
+      <c r="M19"/>
+      <c r="N19" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>754</v>
+      </c>
+      <c r="B20" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C20" t="s">
+        <v>755</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="s">
+        <v>756</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20"/>
+      <c r="K20"/>
+      <c r="L20"/>
+      <c r="M20"/>
+      <c r="N20" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>757</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C21" t="s">
+        <v>758</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>759</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21"/>
+      <c r="K21"/>
+      <c r="L21"/>
+      <c r="M21"/>
+      <c r="N21" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>760</v>
+      </c>
+      <c r="B22" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C22" t="s">
+        <v>761</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="s">
+        <v>762</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22"/>
+      <c r="K22"/>
+      <c r="L22"/>
+      <c r="M22"/>
+      <c r="N22" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>763</v>
+      </c>
+      <c r="B23" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C23" t="s">
+        <v>764</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>765</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23"/>
+      <c r="K23"/>
+      <c r="L23"/>
+      <c r="M23"/>
+      <c r="N23" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>766</v>
+      </c>
+      <c r="B24" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C24" t="s">
+        <v>767</v>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="s">
+        <v>768</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24"/>
+      <c r="K24"/>
+      <c r="L24"/>
+      <c r="M24"/>
+      <c r="N24" t="n">
+        <v>-1.82</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>769</v>
+      </c>
+      <c r="B25" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="C25" t="s">
+        <v>770</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>771</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25"/>
+      <c r="K25"/>
+      <c r="L25"/>
+      <c r="M25"/>
+      <c r="N25" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>772</v>
+      </c>
+      <c r="B26" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>773</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="s">
+        <v>774</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26"/>
+      <c r="K26"/>
+      <c r="L26"/>
+      <c r="M26"/>
+      <c r="N26" t="n">
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>775</v>
+      </c>
+      <c r="B27" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>776</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="s">
+        <v>777</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27"/>
+      <c r="K27"/>
+      <c r="L27"/>
+      <c r="M27" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>778</v>
+      </c>
+      <c r="B28" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C28" t="s">
+        <v>779</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="s">
+        <v>780</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28"/>
+      <c r="K28"/>
+      <c r="L28"/>
+      <c r="M28"/>
+      <c r="N28" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>781</v>
+      </c>
+      <c r="B29" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C29" t="s">
+        <v>782</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="s">
+        <v>783</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29"/>
+      <c r="K29"/>
+      <c r="L29"/>
+      <c r="M29"/>
+      <c r="N29" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>784</v>
+      </c>
+      <c r="B30" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="C30" t="s">
+        <v>785</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="s">
+        <v>786</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30"/>
+      <c r="K30"/>
+      <c r="L30"/>
+      <c r="M30"/>
+      <c r="N30" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>787</v>
+      </c>
+      <c r="B32" t="s">
+        <v>788</v>
+      </c>
+      <c r="C32" t="s">
+        <v>789</v>
+      </c>
+      <c r="D32" t="s">
+        <v>790</v>
+      </c>
+      <c r="E32" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>792</v>
+      </c>
+      <c r="B33" t="s">
+        <v>793</v>
+      </c>
+      <c r="C33" t="s">
+        <v>794</v>
+      </c>
+      <c r="D33" t="s">
+        <v>795</v>
+      </c>
+      <c r="E33" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>797</v>
+      </c>
+      <c r="B34" t="s">
+        <v>798</v>
+      </c>
+      <c r="C34" t="s">
+        <v>799</v>
+      </c>
+      <c r="D34" t="s">
+        <v>800</v>
+      </c>
+      <c r="E34" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>803</v>
+      </c>
+      <c r="B37" t="s">
+        <v>804</v>
+      </c>
+      <c r="C37" t="s">
+        <v>805</v>
+      </c>
+      <c r="D37" t="s">
+        <v>806</v>
+      </c>
+      <c r="E37" t="s">
+        <v>807</v>
+      </c>
+      <c r="F37" t="s">
+        <v>808</v>
+      </c>
+      <c r="G37" t="s">
+        <v>809</v>
+      </c>
+      <c r="H37" t="s">
+        <v>810</v>
+      </c>
+      <c r="I37" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>812</v>
+      </c>
+      <c r="B38" t="s">
+        <v>813</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3</v>
+      </c>
+      <c r="D38" t="s">
+        <v>814</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2</v>
+      </c>
+      <c r="F38" t="s">
+        <v>815</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-0.5</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>816</v>
+      </c>
+      <c r="B39" t="s">
+        <v>817</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="s">
+        <v>818</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" t="s">
+        <v>819</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>1.82</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>820</v>
+      </c>
+      <c r="B40" t="s">
+        <v>821</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="s">
+        <v>822</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="s">
+        <v>823</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>824</v>
+      </c>
+      <c r="B41" t="s">
+        <v>825</v>
+      </c>
+      <c r="C41" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" t="s">
+        <v>826</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" t="s">
+        <v>827</v>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-0.7</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>828</v>
+      </c>
+      <c r="B42" t="s">
+        <v>829</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="s">
+        <v>830</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="s">
+        <v>831</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>832</v>
+      </c>
+      <c r="B43" t="s">
+        <v>833</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="s">
+        <v>834</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="s">
+        <v>835</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>836</v>
+      </c>
+      <c r="B44" t="s">
+        <v>837</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="s">
+        <v>838</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="s">
+        <v>839</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>840</v>
+      </c>
+      <c r="B45" t="s">
+        <v>841</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="s">
+        <v>842</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="s">
+        <v>843</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.91</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>844</v>
+      </c>
+      <c r="B46" t="s">
+        <v>845</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="s">
+        <v>846</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="s">
+        <v>847</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>0.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>